<commit_message>
docs(isa): refresh QEMU support matrix after v0.3 audit
Regenerate from SuperScalarModel tile_profile_status.json; the
bin-20260806 audit evidence is recorded in tile_profile_evidence.json
(bin-20260806_isav03_audit) and cells stay UNVERIFIED without an
independent golden.
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -2652,12 +2652,13 @@
       </c>
       <c r="AR10" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Column-reduce dst published as an LB0-element row/vector tile (TCOLARGMAX.md: one U32 index per column), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AS10" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2880,13 @@
       </c>
       <c r="AR11" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Column-reduce dst published as an LB0-element row/vector tile (TCOLARGMIN.md: one U32 index per column), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AS11" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -4922,12 +4924,13 @@
       </c>
       <c r="AR20" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AS20" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -5149,12 +5152,13 @@
       </c>
       <c r="AR21" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AS21" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -5376,12 +5380,13 @@
       </c>
       <c r="AR22" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AS22" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -5603,12 +5608,13 @@
       </c>
       <c r="AR23" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AS23" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -6057,12 +6063,13 @@
       </c>
       <c r="AR25" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+QEMU TCVT now accepts B.DATR PadValue (Zero/Max/Min/Null) per B.DATR.md PadValue table; the previous TEPL DATR gate rejected PadValue on TCVT. 91-case rerun: tmov/tcvt/cast_back*/expand_to_mhc_bwd/fused_weight/reduce_fused/swiglu PASS. Cell stays UNVERIFIED because bin ELFs are regression material, not independent numeric golden.</t>
         </is>
       </c>
       <c r="AS25" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -13340,12 +13347,13 @@
       </c>
       <c r="AR57" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Zero divisors are data content, not an encoding/descriptor legality condition (TREM.md defines only element-wise remainder with divisor-signed remainder). QEMU no longer rejects divisor tiles containing 0; QEMU returns 0 for zero divisor while gfrun returns all-1s. ISA does not define the zero-divisor value, so the cell stays UNVERIFIED.</t>
         </is>
       </c>
       <c r="AS57" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -13567,12 +13575,13 @@
       </c>
       <c r="AR58" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Zero divisors are data content, not an encoding/descriptor legality condition (TREMS.md defines only element-wise remainder). QEMU no longer rejects divisor tiles containing 0; QEMU returns 0 for zero divisor while gfrun returns all-1s. ISA does not define the zero-divisor value, so the cell stays UNVERIFIED.</t>
         </is>
       </c>
       <c r="AS58" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -21542,12 +21551,13 @@
       </c>
       <c r="AH3" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+MGATHER dst B.DATR PadValue.Null accepted per B.DATR.md PadValue table; index dtype gate enforces S32/U32 per MGATHER.md and fails closed before memory side effects. 91-case rerun: mgather_i32 PASS; mgather_fp16/fp32 and gelu_bf16 FAIL_ILLEGAL because their dst B.DATR DataType=31 is invalid (B.DATR.md), an ELF-side defect. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AI3" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -22073,12 +22083,13 @@
       </c>
       <c r="AH6" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806_isav03_audit
+Source-only stores accept TSize=000 and derive size from the source descriptor per B.IOT.md; index dtype gate enforces S32/U32 per MSCATTER.md and fails closed before memory side effects. 91-case rerun: mscatter_i32 PASS; mscatter_fp16/fp32 FAIL_ILLEGAL because their index tile dtype is FP16/FP32. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
       <c r="AI6" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(isa): mark validated FP32 row/col reduce profiles PASS
Mirror the gfrun support matrix update: TROWSUM/MAX/MIN/PROD and
TCOLSUM/MAX/MIN/PROD (FP32) are PASS on the shared
v5_tepl_reduce_f32_profiles evidence with independent golden.
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -4924,13 +4924,13 @@
       </c>
       <c r="AR20" s="7" t="inlineStr">
         <is>
-          <t>bin-20260806_isav03_audit
-Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -5152,13 +5152,13 @@
       </c>
       <c r="AR21" s="7" t="inlineStr">
         <is>
-          <t>bin-20260806_isav03_audit
-Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -5380,13 +5380,13 @@
       </c>
       <c r="AR22" s="7" t="inlineStr">
         <is>
-          <t>bin-20260806_isav03_audit
-Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -5608,13 +5608,13 @@
       </c>
       <c r="AR23" s="7" t="inlineStr">
         <is>
-          <t>bin-20260806_isav03_audit
-Column-reduce dst published as an LB0-element row/vector tile (TCOLSUM.md: 'dst row/vector tile, one value per column'), no longer gated against the 2D source shape. 91-case rerun: expand_to_mhc_bwd PASS. Cell stays UNVERIFIED without an independent golden.</t>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -16073,12 +16073,13 @@
       </c>
       <c r="AR69" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS69" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -16300,12 +16301,13 @@
       </c>
       <c r="AR70" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS70" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -16527,12 +16529,13 @@
       </c>
       <c r="AR71" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS71" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16757,13 @@
       </c>
       <c r="AR72" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v5_tepl_reduce_f32_profiles
+FP32 row/col reduce of an 8x8 source; TROW* 8x1 column vector with strided LB2=4 destination, TCOL* dense 1x8 row; matches independent sequence golden.</t>
         </is>
       </c>
       <c r="AS72" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(isa): refresh QEMU tile profile matrix after TMOV fix
Adds the Local byte-preserving alias REUSEA/B FP32 profile as PASS for
TMOV, updates TMATMUL_ACC/MGATHER/MSCATTER evidence notes, and marks
TMATMUL_MX UNVERIFIED (ISA defines no MX AType matrix).
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -169,7 +169,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -267,10 +267,10 @@
         <v>3</v>
       </c>
       <c r="D9" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E9" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
@@ -315,10 +315,10 @@
         <v>193</v>
       </c>
       <c r="D11" s="4">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E11" s="5">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
@@ -20804,13 +20804,13 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>v03_group_mma_kchunks3_m16_n32_k16
-Three K chunks prove initial TMATMUL plus repeated explicit-C/D TMATMUL_ACC; every chunk uses SharedTSize class 5, 2 KiB per PE and 8 KiB aggregate.</t>
+          <t>v03_group_mma_kchunks3_m16_n32_k16; bin-20260806 matmul_MASK_MASK_FP32_REUSEA/B
+Canonical Local form B.IOT C,A + B.IOT B,last,-&gt;D validated. bin-20260806 FP16/FP8 MASK_MASK encode (A,B)+(C) non-canonical order and are rejected (fail-closed) per TMATMUL_ACC.md; C must be MxN AccType S32/F32.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -20867,9 +20867,9 @@
           <t>matrix-cube</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>UNSUPPORTED</t>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -20889,13 +20889,13 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>QEMU fail-closed support audit
-The current QEMU head rejects this identity/profile before destination mutation.</t>
+          <t>bin-20260806_isav03_audit; full 356 rerun 2026-08-08
+QEMU MX gate requires AType=FP32 plus e4m3/e5m2 or e2m1x2/HiF4x2 pair; TMATMUL_MX.md does not define the MX AType support matrix, so the 0806 HiF4x2/BF16 MX ELFs stay UNVERIFIED (not counted as model defects).</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -21556,12 +21556,12 @@
       <c r="AH3" s="7" t="inlineStr">
         <is>
           <t>bin-20260806_isav03_audit
-MGATHER dst B.DATR PadValue.Null accepted per B.DATR.md PadValue table; index dtype gate enforces S32/U32 per MGATHER.md and fails closed before memory side effects. 91-case rerun: mgather_i32 PASS; mgather_fp16/fp32 and gelu_bf16 FAIL_ILLEGAL because their dst B.DATR DataType=31 is invalid (B.DATR.md), an ELF-side defect. Cell stays UNVERIFIED without an independent golden.</t>
+B.DATR DataType=31 invalid (B.DATR.md) rejected at decode; index dtype S32/U32 enforced per MGATHER.md before memory side effects. bin-20260806 mgather_i32/fp16/fp32 all FAIL_ILLEGAL (DataType=31 ELF defect). UNVERIFIED without independent golden.</t>
         </is>
       </c>
       <c r="AI3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -22088,12 +22088,12 @@
       <c r="AH6" s="7" t="inlineStr">
         <is>
           <t>bin-20260806_isav03_audit
-Source-only stores accept TSize=000 and derive size from the source descriptor per B.IOT.md; index dtype gate enforces S32/U32 per MSCATTER.md and fails closed before memory side effects. 91-case rerun: mscatter_i32 PASS; mscatter_fp16/fp32 FAIL_ILLEGAL because their index tile dtype is FP16/FP32. Cell stays UNVERIFIED without an independent golden.</t>
+index dtype S32/U32 enforced per MSCATTER.md; mscatter_fp16/fp32 FAIL_ILLEGAL (index FP16/FP32 ELF defect). UNVERIFIED without independent golden.</t>
         </is>
       </c>
       <c r="AI6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -22620,12 +22620,13 @@
       </c>
       <c r="AH9" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>bin-20260806 matmul_MASK_MASK_FP32_REUSEA/B (full 356 rerun); TMOV.md byte-preserving descriptor inheritance fix
+TMOV materialize now inherits the bound source Tile shape for aliased (src==dst) moves; REUSEA/B FP32 flipped FAIL_ILLEGAL -&gt; PASS. Local TMOV with B.IOT dst is legal per TMOV.md; Shared modes (L2S Function 9-12) remain UNVERIFIED here.</t>
         </is>
       </c>
       <c r="AI9" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(linx): rebase PTO v0.58 adaptation onto master
Rebase the reviewed PTO v0.58 QEMU adaptation onto LinxISA master at
c667cdec93ba4ee48bf09c2649c16949e219c95c, preserving Shared TMOV metadata,
shared-left cooperative CUBE, Shared TLOAD/scatter, ADDTPC page semantics,
and the validated contract/regression tests.
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -158,7 +158,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>pto-spec v0.58@3b8cd26c600f0939a143422f175a19cc3ed2999b</t>
+          <t>pto-spec main@4d115387b8a8a3c135f78189778d38547e75c697</t>
         </is>
       </c>
     </row>
@@ -170,7 +170,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -265,17 +265,17 @@
         <v>248</v>
       </c>
       <c r="C9" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D9" s="4">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E9" s="5">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>12.1%</t>
         </is>
       </c>
     </row>
@@ -286,20 +286,20 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" s="4">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
@@ -310,10 +310,10 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C11" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" s="4">
         <v>12</v>
@@ -323,7 +323,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
     </row>
@@ -334,20 +334,20 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="C12" s="3">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D12" s="4">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E12" s="5">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>42.7%</t>
+          <t>43.5%</t>
         </is>
       </c>
     </row>
@@ -379,10 +379,8 @@
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
     <col min="18" max="18" width="14" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="19" max="19" width="58" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="58" customWidth="1"/>
-    <col min="22" max="22" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,40 +456,30 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>F16; output mask: U32</t>
+          <t>FP8/FP4/e8m0; exact pair depends on RoundMode/SaturationMode</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>FP8/FP4/e8m0; exact pair depends on RoundMode/SaturationMode</t>
+          <t>Input: S32</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Input: S32</t>
+          <t>Input: U32</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Input: U32</t>
+          <t>U8/S8/U16/S16/U32/S32/F16/BF16/F32; NORM row-major; 4x32/4x16/4x8; scalar broadcast</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>S16; output mask: U32</t>
+          <t>Evidence / Notes</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>U8/S8/U16/S16/U32/S32/F16/BF16/F32; NORM row-major; 4x32/4x16/4x8; scalar broadcast</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence / Notes</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -588,25 +576,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="S2" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_unary_profiles
 Automated current-ISA profile verification; evidence refs: tabs_f16.</t>
         </is>
       </c>
-      <c r="V2" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T2" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -701,25 +679,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U3" s="7" t="inlineStr">
+      <c r="S3" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_basic_byte_float_profiles; v058_tepl_basic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tadd_u16.</t>
         </is>
       </c>
-      <c r="V3" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -814,25 +782,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U4" s="7" t="inlineStr">
+      <c r="S4" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_arithmetic_byte_float_profiles; v058_tepl_scalar_arithmetic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tadds_u16.</t>
         </is>
       </c>
-      <c r="V4" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -927,25 +885,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U5" s="7" t="inlineStr">
+      <c r="S5" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tand_u16.</t>
         </is>
       </c>
-      <c r="V5" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1040,25 +988,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U6" s="7" t="inlineStr">
+      <c r="S6" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_logical_byte_profiles; v058_tepl_scalar_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tands_u16.</t>
         </is>
       </c>
-      <c r="V6" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1108,9 +1046,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -1133,9 +1071,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
@@ -1143,35 +1081,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="S7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U7" s="7" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S7" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_compare_byte_float_profiles; v058_tepl_compare_integer_profiles
 Automated current-ISA profile verification; evidence refs: tcmp_u16_gt.</t>
         </is>
       </c>
-      <c r="V7" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1201,9 +1129,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1251,14 +1179,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -1266,25 +1194,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U8" s="7" t="inlineStr">
+      <c r="S8" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_compare_scalar_modes; v058_tepl_compare_scalar_profiles
 Automated current-ISA profile verification; evidence refs: tcmps_u16_gt.</t>
         </is>
       </c>
-      <c r="V8" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1359,14 +1277,14 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
@@ -1379,22 +1297,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U9" s="7" t="inlineStr">
+      <c r="S9" s="7" t="inlineStr">
         <is>
           <t>QEMU TCVT now accepts B.DATR PadValue (Zero/Max/Min/Null) per B.DATR.md PadValue table; the previous TEPL DATR gate rejected PadValue on TCVT. 91-case rerun: tmov/tcvt/cast_back*/expand_to_mhc_bwd/fused_weight/reduce_fused/swiglu PASS. Cell stays UNVERIFIED because bin ELFs are regression material, not independent numeric golden.</t>
         </is>
       </c>
-      <c r="V9" s="7" t="inlineStr">
+      <c r="T9" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -1491,22 +1399,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U10" s="7" t="inlineStr">
+      <c r="S10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="V10" s="7" t="inlineStr">
+      <c r="T10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1603,25 +1501,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U11" s="7" t="inlineStr">
+      <c r="S11" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_div_profiles
 Automated current-ISA profile verification; evidence refs: tdivs_f16.</t>
         </is>
       </c>
-      <c r="V11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1711,30 +1599,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T12" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="U12" s="7" t="inlineStr">
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S12" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expands_profiles
 Automated current-ISA profile verification; evidence refs: texpands_u8, texpands_s8, texpands_u16, texpands_s16, texpands_u32, texpands_s32, texpands_f16, texpands_bf16, texpands_f32.</t>
         </is>
       </c>
-      <c r="V12" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1829,25 +1707,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U13" s="7" t="inlineStr">
+      <c r="S13" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tfma_f32
 Automated current-ISA profile verification; evidence refs: tfma_f32.</t>
         </is>
       </c>
-      <c r="V13" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1942,25 +1810,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S14" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T14" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U14" s="7" t="inlineStr">
+      <c r="S14" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_basic_byte_float_profiles; v058_tepl_basic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmax_u16.</t>
         </is>
       </c>
-      <c r="V14" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T14" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2055,25 +1913,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S15" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T15" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U15" s="7" t="inlineStr">
+      <c r="S15" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_minmax_float_profiles; v058_tepl_scalar_minmax_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmaxs_u8.</t>
         </is>
       </c>
-      <c r="V15" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2168,25 +2016,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S16" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T16" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U16" s="7" t="inlineStr">
+      <c r="S16" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_basic_byte_float_profiles; v058_tepl_basic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmin_u16.</t>
         </is>
       </c>
-      <c r="V16" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T16" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2281,25 +2119,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S17" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T17" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U17" s="7" t="inlineStr">
+      <c r="S17" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_minmax_float_profiles; v058_tepl_scalar_minmax_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmins_u8.</t>
         </is>
       </c>
-      <c r="V17" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2394,25 +2222,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S18" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T18" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U18" s="7" t="inlineStr">
+      <c r="S18" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sub_mul_byte_float_profiles; v058_tepl_sub_mul_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmul_u16.</t>
         </is>
       </c>
-      <c r="V18" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T18" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2507,25 +2325,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S19" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T19" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U19" s="7" t="inlineStr">
+      <c r="S19" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_arithmetic_byte_float_profiles; v058_tepl_scalar_arithmetic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tmuls_u16.</t>
         </is>
       </c>
-      <c r="V19" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T19" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2620,25 +2428,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U20" s="7" t="inlineStr">
+      <c r="S20" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_unary_profiles
 Automated current-ISA profile verification; evidence refs: tneg_bf16.</t>
         </is>
       </c>
-      <c r="V20" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T20" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2733,25 +2531,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S21" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T21" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U21" s="7" t="inlineStr">
+      <c r="S21" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tnot_u16.</t>
         </is>
       </c>
-      <c r="V21" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2846,25 +2634,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U22" s="7" t="inlineStr">
+      <c r="S22" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tor_u16.</t>
         </is>
       </c>
-      <c r="V22" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2959,25 +2737,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U23" s="7" t="inlineStr">
+      <c r="S23" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_logical_byte_profiles; v058_tepl_scalar_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tors_u16.</t>
         </is>
       </c>
-      <c r="V23" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -3072,25 +2840,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S24" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T24" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U24" s="7" t="inlineStr">
+      <c r="S24" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_unary_profiles
 Automated current-ISA profile verification; evidence refs: trelu_s32.</t>
         </is>
       </c>
-      <c r="V24" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T24" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -3185,22 +2943,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U25" s="7" t="inlineStr">
+      <c r="S25" s="7" t="inlineStr">
         <is>
           <t>Zero divisors are data content, not an encoding/descriptor legality condition (TREM.md defines only element-wise remainder with divisor-signed remainder). QEMU no longer rejects divisor tiles containing 0; QEMU returns 0 for zero divisor while gfrun returns all-1s. ISA does not define the zero-divisor value, so the cell stays UNVERIFIED.</t>
         </is>
       </c>
-      <c r="V25" s="7" t="inlineStr">
+      <c r="T25" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -3297,22 +3045,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S26" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T26" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U26" s="7" t="inlineStr">
+      <c r="S26" s="7" t="inlineStr">
         <is>
           <t>Zero divisors are data content, not an encoding/descriptor legality condition (TREMS.md defines only element-wise remainder). QEMU no longer rejects divisor tiles containing 0; QEMU returns 0 for zero divisor while gfrun returns all-1s. ISA does not define the zero-divisor value, so the cell stays UNVERIFIED.</t>
         </is>
       </c>
-      <c r="V26" s="7" t="inlineStr">
+      <c r="T26" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -3409,25 +3147,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S27" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T27" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U27" s="7" t="inlineStr">
+      <c r="S27" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_select_byte_profiles; v058_tepl_select_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tsel_s16.</t>
         </is>
       </c>
-      <c r="V27" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -3522,25 +3250,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S28" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T28" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U28" s="7" t="inlineStr">
+      <c r="S28" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_select_byte_profiles; v058_tepl_select_word_half_profiles
 Automated current-ISA profile verification; evidence refs: tsels_u16.</t>
         </is>
       </c>
-      <c r="V28" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T28" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -3635,25 +3353,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S29" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T29" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U29" s="7" t="inlineStr">
+      <c r="S29" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshl_u8.</t>
         </is>
       </c>
-      <c r="V29" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -3748,25 +3456,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S30" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T30" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U30" s="7" t="inlineStr">
+      <c r="S30" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshls_u8.</t>
         </is>
       </c>
-      <c r="V30" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T30" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -3861,25 +3559,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S31" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T31" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U31" s="7" t="inlineStr">
+      <c r="S31" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshr_u8.</t>
         </is>
       </c>
-      <c r="V31" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -3974,25 +3662,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S32" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T32" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U32" s="7" t="inlineStr">
+      <c r="S32" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_shift_profiles
 Automated current-ISA profile verification; evidence refs: tshrs_u8.</t>
         </is>
       </c>
-      <c r="V32" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T32" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4087,25 +3765,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S33" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T33" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U33" s="7" t="inlineStr">
+      <c r="S33" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sub_mul_byte_float_profiles; v058_tepl_sub_mul_integer_profiles
 Automated current-ISA profile verification; evidence refs: tsub_u16.</t>
         </is>
       </c>
-      <c r="V33" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T33" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4200,25 +3868,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S34" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T34" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U34" s="7" t="inlineStr">
+      <c r="S34" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_arithmetic_byte_float_profiles; v058_tepl_scalar_arithmetic_integer_profiles
 Automated current-ISA profile verification; evidence refs: tsubs_s16.</t>
         </is>
       </c>
-      <c r="V34" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T34" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4313,25 +3971,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S35" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T35" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U35" s="7" t="inlineStr">
+      <c r="S35" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_logical_byte_profiles; v058_tepl_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: txor_u16.</t>
         </is>
       </c>
-      <c r="V35" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T35" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4426,30 +4074,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S36" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T36" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U36" s="7" t="inlineStr">
+      <c r="S36" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_scalar_logical_byte_profiles; v058_tepl_scalar_logical_word_half_profiles
 Automated current-ISA profile verification; evidence refs: txors_u16.</t>
         </is>
       </c>
-      <c r="V36" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="T36" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V36"/>
+  <autoFilter ref="A1:T36"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -4879,7 +4517,7 @@
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5094,7 @@
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -6993,7 +6631,7 @@
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -7186,7 +6824,7 @@
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7017,7 @@
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7210,7 @@
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -8208,9 +7846,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
@@ -8335,12 +7973,13 @@
       </c>
       <c r="AK20" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_irregular_layout_profiles
+Automated current-ISA profile verification; evidence refs: textract_fp32.</t>
         </is>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -8769,121 +8408,121 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="X23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Y23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AB23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AC23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AD23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE23" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="P23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="V23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Z23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AB23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AC23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AD23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AE23" s="5" t="inlineStr">
-        <is>
-          <t>UNSUPPORTED</t>
-        </is>
-      </c>
       <c r="AF23" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -8911,13 +8550,13 @@
       </c>
       <c r="AK23" s="7" t="inlineStr">
         <is>
-          <t>QEMU fail-closed support audit
-The current QEMU head rejects this identity/profile before destination mutation.</t>
+          <t>v058_irregular_layout_profiles
+Automated current-ISA profile verification; evidence refs: thistogram_u32_byte3.</t>
         </is>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -11418,7 +11057,7 @@
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -12955,7 +12594,7 @@
       </c>
       <c r="AL44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -13148,7 +12787,7 @@
       </c>
       <c r="AL45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -13341,7 +12980,7 @@
       </c>
       <c r="AL46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -13534,7 +13173,7 @@
       </c>
       <c r="AL47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -14687,7 +14326,7 @@
       </c>
       <c r="AL53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -14736,8 +14375,9 @@
     <col min="33" max="33" width="14" customWidth="1"/>
     <col min="34" max="34" width="14" customWidth="1"/>
     <col min="35" max="35" width="14" customWidth="1"/>
-    <col min="36" max="36" width="58" customWidth="1"/>
-    <col min="37" max="37" width="14" customWidth="1"/>
+    <col min="36" max="36" width="14" customWidth="1"/>
+    <col min="37" max="37" width="58" customWidth="1"/>
+    <col min="38" max="38" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14803,125 +14443,130 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Local FP16; valid 4x16; NORM row-major; PE-local 128B</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Local FP32; 16x16; NORM row-major; PE-local 1KiB</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 16x32; NORM row-major; PE-local 2KiB</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 32x32; NORM row-major; PE-local 4KiB</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 8x16; NORM row-major; PE-local 512B</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Local FP32; 8x32; NORM row-major; PE-local 1KiB</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Local NORM S8/U8/S16/U16/S32/U32/F32; logical row stride; valid rectangle</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Local S32; valid 4x8; NORM row-major; PE-local 128B</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>PTO TLOAD dtype/layout combinations supported by the v5 TLSU profile</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>PTO TSTORE dtype/layout combinations supported by the v5 TLSU profile</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Same element dtype set as TLOAD profile; src/dst element size must match</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K16xN32 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K32xN16 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K32xN32 NORM; PE-local 4KiB class 6; Core4 aggregate 16KiB</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Shared full S8; PE0 issuer; K16xN32 NORM; PE-local 512B class 3; Core4 aggregate 2KiB</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Shared full/core FP32; B.IOS source; Function 1; NORM</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Shared pe_scope FP32; B.IOS source; Function 14; NORM</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>TLSU atomic data types accepted by BSTART.MGATHER.CAS</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>TLSU data types accepted by BSTART.MGATHER.MASK</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>TLSU data types accepted by BSTART.MSCATTER.MASK</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>byte-preserving; descriptors must be compatible</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>byte-preserving; source and destination descriptors must match</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>data: S8</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>data: U8</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Evidence / Notes</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -15088,28 +14733,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AG2" s="5" t="inlineStr">
+      <c r="AG2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AH2" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="AH2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AI2" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ2" s="7" t="inlineStr">
+      <c r="AJ2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK2" s="7" t="inlineStr">
         <is>
           <t>QEMU fail-closed support audit
 The current QEMU head rejects this identity/profile before destination mutation.</t>
         </is>
       </c>
-      <c r="AK2" s="7" t="inlineStr">
+      <c r="AL2" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15156,9 +14806,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -15286,19 +14936,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AJ3" s="7" t="inlineStr">
-        <is>
-          <t>MGATHER dst B.DATR PadValue.Null accepted per B.DATR.md PadValue table; index dtype gate enforces S32/U32 per MGATHER.md and fails closed before memory side effects. 91-case rerun: mgather_i32 PASS; mgather_fp16/fp32 and gelu_bf16 FAIL_ILLEGAL because their dst B.DATR DataType=31 is invalid (B.DATR.md), an ELF-side defect. Cell stays UNVERIFIED without an independent golden.</t>
+      <c r="AI3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ3" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AK3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>v058_irregular_layout_profiles
+Automated current-ISA profile verification; evidence refs: mgather_u32.</t>
+        </is>
+      </c>
+      <c r="AL3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -15443,14 +15099,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AC4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AD4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AC4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AD4" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AE4" s="6" t="inlineStr">
@@ -15478,12 +15134,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ4" s="7" t="inlineStr">
+      <c r="AJ4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK4" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK4" s="7" t="inlineStr">
+      <c r="AL4" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15635,14 +15296,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AD5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AE5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AD5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE5" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AF5" s="6" t="inlineStr">
@@ -15665,12 +15326,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ5" s="7" t="inlineStr">
+      <c r="AJ5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK5" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK5" s="7" t="inlineStr">
+      <c r="AL5" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15842,22 +15508,27 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AI6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ6" s="7" t="inlineStr">
+      <c r="AH6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AI6" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AJ6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK6" s="7" t="inlineStr">
         <is>
           <t>Source-only stores accept TSize=000 and derive size from the source descriptor per B.IOT.md; index dtype gate enforces S32/U32 per MSCATTER.md and fails closed before memory side effects. 91-case rerun: mscatter_i32 PASS; mscatter_fp16/fp32 FAIL_ILLEGAL because their index tile dtype is FP16/FP32. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
-      <c r="AK6" s="7" t="inlineStr">
+      <c r="AL6" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -16014,14 +15685,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AE7" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AF7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AE7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AF7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AG7" s="6" t="inlineStr">
@@ -16039,12 +15710,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ7" s="7" t="inlineStr">
+      <c r="AJ7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK7" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK7" s="7" t="inlineStr">
+      <c r="AL7" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -16111,34 +15787,34 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="P8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
@@ -16146,14 +15822,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="U8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="V8" s="6" t="inlineStr">
@@ -16161,9 +15837,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="W8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="X8" s="4" t="inlineStr">
@@ -16181,9 +15857,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AA8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AA8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AB8" s="6" t="inlineStr">
@@ -16226,15 +15902,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ8" s="7" t="inlineStr">
-        <is>
-          <t>v058_tload_tile_state; v058_tload_tstore_common_profiles
+      <c r="AJ8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK8" s="7" t="inlineStr">
+        <is>
+          <t>v058_tload_fp16_tile_state; v058_tload_tile_state; v058_tload_tstore_common_profiles
 Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_row1, s16_row0, s16_row1, s8_row0, s8_row1, u8_row0, u8_row1, u16_row0, u16_row1, s32_row0, s32_row1, u32_row0, u32_row1, zero_stride_rows.</t>
         </is>
       </c>
-      <c r="AK8" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="AL8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -16394,14 +16075,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AF9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AG9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AF9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AG9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AH9" s="6" t="inlineStr">
@@ -16414,13 +16095,18 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ9" s="7" t="inlineStr">
+      <c r="AJ9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK9" s="7" t="inlineStr">
         <is>
           <t>bin-20260806 matmul_MASK_MASK_FP32_REUSEA/B (full 356 rerun); TMOV.md byte-preserving descriptor inheritance fix
 TMOV materialize now inherits the bound source Tile shape for aliased (src==dst) moves; REUSEA/B FP32 flipped FAIL_ILLEGAL -&gt; PASS. Local TMOV with B.IOT dst is legal per TMOV.md; Shared modes (L2S Function 9-12) remain UNVERIFIED here.</t>
         </is>
       </c>
-      <c r="AK9" s="7" t="inlineStr">
+      <c r="AL9" s="7" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
@@ -16532,14 +16218,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="W10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="X10" s="6" t="inlineStr">
@@ -16602,12 +16288,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ10" s="7" t="inlineStr">
+      <c r="AJ10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AK10" s="7" t="inlineStr">
+      <c r="AL10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -16679,9 +16370,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
@@ -16694,34 +16385,34 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="Q11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="S11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="T11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="V11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="W11" s="6" t="inlineStr">
@@ -16744,9 +16435,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AA11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AA11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AB11" s="3" t="inlineStr">
@@ -16754,9 +16445,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="AC11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AC11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AD11" s="6" t="inlineStr">
@@ -16789,20 +16480,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ11" s="7" t="inlineStr">
+      <c r="AJ11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK11" s="7" t="inlineStr">
         <is>
           <t>v058_shared_tlsu; v058_tload_tstore_common_profiles
-Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_row1, s16_row0, s16_row1, s8_row0, s8_row1, u8_row0, u8_row1, u16_row0, u16_row1, s32_row0, s32_row1, u32_row0, u32_row1, zero_stride_rows.</t>
-        </is>
-      </c>
-      <c r="AK11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+Automated current-ISA profile verification; evidence refs: shared_part_pe0, shared_part_pe1, shared_part_pe2, shared_part_pe3.</t>
+        </is>
+      </c>
+      <c r="AL11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK11"/>
+  <autoFilter ref="A1:AL11"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -16827,8 +16523,9 @@
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="58" customWidth="1"/>
-    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="18" max="18" width="58" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16914,10 +16611,15 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>Shared Left F32xF32 + Shared Right F32xF32 -&gt; Local F32 D; NORM; Core4; M=N=K=32; 4KB per PE</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Evidence / Notes</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -17004,15 +16706,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q2" s="7" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R2" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_s32_m4_k4_col8.</t>
         </is>
       </c>
-      <c r="R2" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S2" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17097,15 +16804,20 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="Q3" s="7" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R3" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_acc_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_acc_s32_m4_k4_explicit_c.</t>
         </is>
       </c>
-      <c r="R3" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17190,15 +16902,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q4" s="7" t="inlineStr">
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R4" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_bias_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_bias_s32_m4_k4_scalar_bias.</t>
         </is>
       </c>
-      <c r="R4" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S4" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17283,15 +17000,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q5" s="7" t="inlineStr">
+      <c r="Q5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R5" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_e4m3_m4_k4.</t>
         </is>
       </c>
-      <c r="R5" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17376,15 +17098,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q6" s="7" t="inlineStr">
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R6" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_acc_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_acc_e4m3_explicit_c.</t>
         </is>
       </c>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17469,15 +17196,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q7" s="7" t="inlineStr">
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R7" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_bias_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_bias_e4m3_scalar_bias.</t>
         </is>
       </c>
-      <c r="R7" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17562,15 +17294,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q8" s="7" t="inlineStr">
-        <is>
-          <t>v058_cube_tmatmul_s32
-Automated current-ISA profile verification; evidence refs: single_tmatmul_s32_m4_n8_k4_col8.</t>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>v058_cube_tmatmul_s32; v058_cube_tmatmul_shared_ab_fp32
+Automated current-ISA profile verification; evidence refs: shared_ab_tmatmul_fp32_m32_n32_k32.</t>
+        </is>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17655,15 +17392,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q9" s="7" t="inlineStr">
+      <c r="Q9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R9" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_acc_s32
 Automated current-ISA profile verification; evidence refs: single_tmatmul_acc_s32_m4_n8_k4_explicit_c.</t>
         </is>
       </c>
-      <c r="R9" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S9" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17748,15 +17490,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q10" s="7" t="inlineStr">
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R10" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_bias_s32
 Automated current-ISA profile verification; evidence refs: single_tmatmul_bias_s32_m4_n8_k4_row_bias.</t>
         </is>
       </c>
-      <c r="R10" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17841,15 +17588,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q11" s="7" t="inlineStr">
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R11" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_e4m3_m4_n8_k4.</t>
         </is>
       </c>
-      <c r="R11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -17934,15 +17686,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q12" s="7" t="inlineStr">
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R12" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_acc_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_acc_e4m3_explicit_c.</t>
         </is>
       </c>
-      <c r="R12" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S12" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -18027,20 +17784,25 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q13" s="7" t="inlineStr">
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R13" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_bias_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_bias_e4m3_row_bias.</t>
         </is>
       </c>
-      <c r="R13" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R13"/>
+  <autoFilter ref="A1:S13"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: refresh QEMU tile profile matrix
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -170,7 +170,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -286,10 +286,10 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C10" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D10" s="4">
         <v>35</v>
@@ -299,7 +299,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>23.4%</t>
         </is>
       </c>
     </row>
@@ -334,10 +334,10 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C12" s="3">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D12" s="4">
         <v>280</v>
@@ -347,7 +347,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>43.9%</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="T2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="T3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="T4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="T20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="T22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="T24" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
       </c>
       <c r="T30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
       </c>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3670,7 @@
       </c>
       <c r="T32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="T34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="T36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4517,7 @@
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -7017,7 +7017,7 @@
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -8556,7 +8556,7 @@
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -11057,7 +11057,7 @@
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -12594,7 +12594,7 @@
       </c>
       <c r="AL44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="AL45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -12980,7 +12980,7 @@
       </c>
       <c r="AL46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="AL47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -14326,7 +14326,7 @@
       </c>
       <c r="AL53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -14376,8 +14376,12 @@
     <col min="34" max="34" width="14" customWidth="1"/>
     <col min="35" max="35" width="14" customWidth="1"/>
     <col min="36" max="36" width="14" customWidth="1"/>
-    <col min="37" max="37" width="58" customWidth="1"/>
+    <col min="37" max="37" width="14" customWidth="1"/>
     <col min="38" max="38" width="14" customWidth="1"/>
+    <col min="39" max="39" width="14" customWidth="1"/>
+    <col min="40" max="40" width="14" customWidth="1"/>
+    <col min="41" max="41" width="58" customWidth="1"/>
+    <col min="42" max="42" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14498,75 +14502,95 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
+          <t>Shared FP32; Function 10 L2S PUBLISH; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Shared FP32; Function 11 S2L BROADCAST; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Shared FP32; Function 12 S2L EXTRACT; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Shared FP32; Function 9 L2S INSERT; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>Shared full FP32; PE0 issuer; K16xN32 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K32xN16 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Shared full FP32; PE0 issuer; K32xN32 NORM; PE-local 4KiB class 6; Core4 aggregate 16KiB</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Shared full S8; PE0 issuer; K16xN32 NORM; PE-local 512B class 3; Core4 aggregate 2KiB</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Shared full/core FP32; B.IOS source; Function 1; NORM</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Shared pe_scope FP32; B.IOS source; Function 14; NORM</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>TLSU atomic data types accepted by BSTART.MGATHER.CAS</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>TLSU data types accepted by BSTART.MGATHER.MASK</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>TLSU data types accepted by BSTART.MSCATTER.MASK</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>byte-preserving; descriptors must be compatible</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>byte-preserving; source and destination descriptors must match</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>data: S8</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>data: U8</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Evidence / Notes</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -14738,28 +14762,48 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH2" s="5" t="inlineStr">
+      <c r="AH2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AI2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL2" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="AI2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK2" s="7" t="inlineStr">
+      <c r="AM2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO2" s="7" t="inlineStr">
         <is>
           <t>QEMU fail-closed support audit
 The current QEMU head rejects this identity/profile before destination mutation.</t>
         </is>
       </c>
-      <c r="AL2" s="7" t="inlineStr">
+      <c r="AP2" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -14941,20 +14985,40 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AK3" s="7" t="inlineStr">
+      <c r="AJ3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN3" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AO3" s="7" t="inlineStr">
         <is>
           <t>v058_irregular_layout_profiles
 Automated current-ISA profile verification; evidence refs: mgather_u32.</t>
         </is>
       </c>
-      <c r="AL3" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
+      <c r="AP3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -15104,9 +15168,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AD4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AD4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AE4" s="6" t="inlineStr">
@@ -15124,9 +15188,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AH4" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AI4" s="6" t="inlineStr">
@@ -15139,12 +15203,32 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK4" s="7" t="inlineStr">
+      <c r="AK4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO4" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AL4" s="7" t="inlineStr">
+      <c r="AP4" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15301,9 +15385,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AE5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AE5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AF5" s="6" t="inlineStr">
@@ -15321,9 +15405,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AI5" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AJ5" s="6" t="inlineStr">
@@ -15331,12 +15415,32 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK5" s="7" t="inlineStr">
+      <c r="AK5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO5" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AL5" s="7" t="inlineStr">
+      <c r="AP5" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15513,9 +15617,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AI6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AJ6" s="6" t="inlineStr">
@@ -15523,12 +15627,32 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK6" s="7" t="inlineStr">
+      <c r="AK6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM6" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AN6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO6" s="7" t="inlineStr">
         <is>
           <t>Source-only stores accept TSize=000 and derive size from the source descriptor per B.IOT.md; index dtype gate enforces S32/U32 per MSCATTER.md and fails closed before memory side effects. 91-case rerun: mscatter_i32 PASS; mscatter_fp16/fp32 FAIL_ILLEGAL because their index tile dtype is FP16/FP32. Cell stays UNVERIFIED without an independent golden.</t>
         </is>
       </c>
-      <c r="AL6" s="7" t="inlineStr">
+      <c r="AP6" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -15690,9 +15814,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AF7" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AF7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AG7" s="6" t="inlineStr">
@@ -15710,17 +15834,37 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK7" s="7" t="inlineStr">
+      <c r="AJ7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AK7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO7" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AL7" s="7" t="inlineStr">
+      <c r="AP7" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -15842,44 +15986,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="Y8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="Z8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AA8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AB8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AC8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AD8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AE8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="X8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Y8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AB8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AC8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AD8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AE8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="AF8" s="6" t="inlineStr">
@@ -15907,15 +16051,35 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK8" s="7" t="inlineStr">
+      <c r="AK8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO8" s="7" t="inlineStr">
         <is>
           <t>v058_tload_fp16_tile_state; v058_tload_tile_state; v058_tload_tstore_common_profiles
 Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_row1, s16_row0, s16_row1, s8_row0, s8_row1, u8_row0, u8_row1, u16_row0, u16_row1, s32_row0, s32_row1, u32_row0, u32_row1, zero_stride_rows.</t>
         </is>
       </c>
-      <c r="AL8" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
+      <c r="AP8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -16035,24 +16199,24 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="X9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Y9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Z9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="X9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AB9" s="6" t="inlineStr">
@@ -16080,9 +16244,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AG9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AG9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AH9" s="6" t="inlineStr">
@@ -16100,15 +16264,35 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK9" s="7" t="inlineStr">
-        <is>
-          <t>bin-20260806 matmul_MASK_MASK_FP32_REUSEA/B (full 356 rerun); TMOV.md byte-preserving descriptor inheritance fix
-TMOV materialize now inherits the bound source Tile shape for aliased (src==dst) moves; REUSEA/B FP32 flipped FAIL_ILLEGAL -&gt; PASS. Local TMOV with B.IOT dst is legal per TMOV.md; Shared modes (L2S Function 9-12) remain UNVERIFIED here.</t>
-        </is>
-      </c>
-      <c r="AL9" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
+      <c r="AK9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="AL9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO9" s="7" t="inlineStr">
+        <is>
+          <t>v058_tmov_shared_fp32
+Automated current-ISA profile verification; evidence refs: publish_extract_pe0, publish_extract_pe1, publish_extract_pe2, publish_extract_pe3.</t>
+        </is>
+      </c>
+      <c r="AP9" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -16293,12 +16477,32 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK10" s="7" t="inlineStr">
+      <c r="AK10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AL10" s="7" t="inlineStr">
+      <c r="AP10" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -16440,14 +16644,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AB11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AC11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AB11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AC11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AD11" s="6" t="inlineStr">
@@ -16460,14 +16664,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AF11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AF11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AH11" s="6" t="inlineStr">
@@ -16485,20 +16689,40 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK11" s="7" t="inlineStr">
+      <c r="AK11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO11" s="7" t="inlineStr">
         <is>
           <t>v058_shared_tlsu; v058_tload_tstore_common_profiles
 Automated current-ISA profile verification; evidence refs: shared_part_pe0, shared_part_pe1, shared_part_pe2, shared_part_pe3.</t>
         </is>
       </c>
-      <c r="AL11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
+      <c r="AP11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AL11"/>
+  <autoFilter ref="A1:AP11"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -16719,7 +16943,7 @@
       </c>
       <c r="S2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -16817,7 +17041,7 @@
       </c>
       <c r="S3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -16915,7 +17139,7 @@
       </c>
       <c r="S4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17013,7 +17237,7 @@
       </c>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17111,7 +17335,7 @@
       </c>
       <c r="S6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17209,7 +17433,7 @@
       </c>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17307,7 +17531,7 @@
       </c>
       <c r="S8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17405,7 +17629,7 @@
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17503,7 +17727,7 @@
       </c>
       <c r="S10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17601,7 +17825,7 @@
       </c>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17699,7 +17923,7 @@
       </c>
       <c r="S12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -17797,7 +18021,7 @@
       </c>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(linx): align PTO identity and FP4 MX contract
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -310,10 +310,10 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C11" s="3">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D11" s="4">
         <v>12</v>
@@ -323,7 +323,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>58.6%</t>
         </is>
       </c>
     </row>
@@ -334,10 +334,10 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="C12" s="3">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D12" s="4">
         <v>280</v>
@@ -347,7 +347,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>43.9%</t>
+          <t>44.3%</t>
         </is>
       </c>
     </row>
@@ -16748,8 +16748,12 @@
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
-    <col min="18" max="18" width="58" customWidth="1"/>
+    <col min="18" max="18" width="14" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="14" customWidth="1"/>
+    <col min="22" max="22" width="58" customWidth="1"/>
+    <col min="23" max="23" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16775,75 +16779,95 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Local E2M1X2xE2M1X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Local E2M1X2xHiF4X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Local E4M3 matrix/vector with E8M0 scales + scalar FP32 bias -&gt; F32; M4N1K4</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Local E4M3 matrix/vector with E8M0 scales -&gt; F32; M4N1K4; Col8</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Local E4M3xE4M3 with E8M0 scales + FP32 row bias -&gt; F32; M4N8K4</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Local E4M3xE4M3 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Local HiF4X2xE2M1X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Local HiF4X2xHiF4X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Local S32 matrix x S32 vector + scalar S32 bias -&gt; S32; M4N1K4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Local S32 matrix x S32 vector -&gt; S32; NORM; M4N1K4; Col8</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Local S32xS32 + row-bias S32 -&gt; S32; NORM; M4N8K4; Col8</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Local S32xS32 -&gt; S32; NORM row-major; M4N8K4; Col8; 256B D</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Local explicit C S32 + S32xS32 -&gt; S32 D; NORM; M4N8K4; Col8</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Local explicit FP32 C + E4M3 matrix/vector with E8M0 scales -&gt; F32 D; M4N1K4</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Local explicit FP32 C + E4M3xE4M3 with E8M0 scales -&gt; F32 D; M4N8K4</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Local explicit S32 C + S32 matrix x vector -&gt; S32 D; M4N1K4; Col8</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Shared Left F32xF32 + Shared Right F32xF32 -&gt; Local F32 D; NORM; Core4; M=N=K=32; 4KB per PE</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Evidence / Notes</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -16895,9 +16919,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -16915,9 +16939,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O2" s="6" t="inlineStr">
@@ -16935,13 +16959,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V2" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_s32_m4_k4_col8.</t>
         </is>
       </c>
-      <c r="S2" s="7" t="inlineStr">
+      <c r="W2" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17023,9 +17067,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="Q3" s="6" t="inlineStr">
@@ -17033,13 +17077,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R3" s="7" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V3" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_acc_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_acc_s32_m4_k4_explicit_c.</t>
         </is>
       </c>
-      <c r="S3" s="7" t="inlineStr">
+      <c r="W3" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17086,9 +17150,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -17106,9 +17170,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -17131,13 +17195,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R4" s="7" t="inlineStr">
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V4" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_bias_s32
 Automated current-ISA profile verification; evidence refs: single_tgemv_bias_s32_m4_k4_scalar_bias.</t>
         </is>
       </c>
-      <c r="S4" s="7" t="inlineStr">
+      <c r="W4" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17169,9 +17253,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -17179,9 +17263,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -17229,13 +17313,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R5" s="7" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V5" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_e4m3_m4_k4.</t>
         </is>
       </c>
-      <c r="S5" s="7" t="inlineStr">
+      <c r="W5" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17307,9 +17411,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -17327,13 +17431,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R6" s="7" t="inlineStr">
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V6" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_acc_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_acc_e4m3_explicit_c.</t>
         </is>
       </c>
-      <c r="S6" s="7" t="inlineStr">
+      <c r="W6" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17360,9 +17484,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -17370,9 +17494,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -17425,13 +17549,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R7" s="7" t="inlineStr">
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V7" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tgemv_mx_bias_e4m3
 Automated current-ISA profile verification; evidence refs: single_tgemv_mx_bias_e4m3_scalar_bias.</t>
         </is>
       </c>
-      <c r="S7" s="7" t="inlineStr">
+      <c r="W7" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17493,9 +17637,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -17513,23 +17657,43 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="R8" s="7" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V8" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_s32; v058_cube_tmatmul_shared_ab_fp32
 Automated current-ISA profile verification; evidence refs: shared_ab_tmatmul_fp32_m32_n32_k32.</t>
         </is>
       </c>
-      <c r="S8" s="7" t="inlineStr">
+      <c r="W8" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17596,9 +17760,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
@@ -17616,18 +17780,38 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R9" s="7" t="inlineStr">
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V9" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_acc_s32
 Automated current-ISA profile verification; evidence refs: single_tmatmul_acc_s32_m4_n8_k4_explicit_c.</t>
         </is>
       </c>
-      <c r="S9" s="7" t="inlineStr">
+      <c r="W9" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17684,9 +17868,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -17704,9 +17888,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P10" s="6" t="inlineStr">
@@ -17719,13 +17903,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R10" s="7" t="inlineStr">
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V10" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_bias_s32
 Automated current-ISA profile verification; evidence refs: single_tmatmul_bias_s32_m4_n8_k4_row_bias.</t>
         </is>
       </c>
-      <c r="S10" s="7" t="inlineStr">
+      <c r="W10" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17752,14 +17956,14 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -17767,9 +17971,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -17777,19 +17981,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
@@ -17817,13 +18021,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R11" s="7" t="inlineStr">
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V11" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_e4m3_m4_n8_k4.</t>
         </is>
       </c>
-      <c r="S11" s="7" t="inlineStr">
+      <c r="W11" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17900,9 +18124,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P12" s="6" t="inlineStr">
@@ -17915,13 +18139,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R12" s="7" t="inlineStr">
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V12" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_acc_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_acc_e4m3_explicit_c.</t>
         </is>
       </c>
-      <c r="S12" s="7" t="inlineStr">
+      <c r="W12" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -17958,9 +18202,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -17968,9 +18212,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -18013,20 +18257,40 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R13" s="7" t="inlineStr">
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V13" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_mx_bias_e4m3
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_bias_e4m3_row_bias.</t>
         </is>
       </c>
-      <c r="S13" s="7" t="inlineStr">
+      <c r="W13" s="7" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S13"/>
+  <autoFilter ref="A1:W13"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(qemu): refresh tile profile support matrix
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -158,7 +158,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>pto-spec main@4d115387b8a8a3c135f78189778d38547e75c697</t>
+          <t>pto-spec 4d115387b8a8a3c135f78189778d38547e75c697@4d115387b8a8a3c135f78189778d38547e75c697</t>
         </is>
       </c>
     </row>
@@ -170,7 +170,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -241,17 +241,17 @@
         <v>222</v>
       </c>
       <c r="C8" s="3">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="D8" s="4">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E8" s="5">
         <v>2</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>82.9%</t>
+          <t>85.6%</t>
         </is>
       </c>
     </row>
@@ -289,17 +289,17 @@
         <v>47</v>
       </c>
       <c r="C10" s="3">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D10" s="4">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>38.3%</t>
         </is>
       </c>
     </row>
@@ -337,17 +337,17 @@
         <v>546</v>
       </c>
       <c r="C12" s="3">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="D12" s="4">
-        <v>280</v>
+        <v>267</v>
       </c>
       <c r="E12" s="5">
         <v>24</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>44.3%</t>
+          <t>46.7%</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="T2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="T3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="T4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="T20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="T22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="T24" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3077,9 +3077,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -3087,9 +3087,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -3097,9 +3097,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -3149,13 +3149,13 @@
       </c>
       <c r="S27" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_select_byte_profiles; v058_tepl_select_word_half_profiles
-Automated current-ISA profile verification; evidence refs: tsel_s16.</t>
+          <t>v058_tepl_select_byte_profiles; v058_tepl_select_complementary_profiles; v058_tepl_select_word_half_profiles
+Automated current-ISA profile verification; evidence refs: tsel_u8.</t>
         </is>
       </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3175,9 +3175,9 @@
           <t>tile-scalar-and-immediate-logical</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -3185,9 +3185,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -3195,9 +3195,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -3252,13 +3252,13 @@
       </c>
       <c r="S28" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_select_byte_profiles; v058_tepl_select_word_half_profiles
-Automated current-ISA profile verification; evidence refs: tsels_u16.</t>
+          <t>v058_tepl_select_byte_profiles; v058_tepl_select_complementary_profiles; v058_tepl_select_word_half_profiles
+Automated current-ISA profile verification; evidence refs: tsels_s8.</t>
         </is>
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
       </c>
       <c r="T30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
       </c>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3670,7 @@
       </c>
       <c r="T32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="T34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="T36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4517,7 @@
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -7017,7 +7017,7 @@
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -8556,7 +8556,7 @@
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -11057,7 +11057,7 @@
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -12594,7 +12594,7 @@
       </c>
       <c r="AL44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="AL45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -12980,7 +12980,7 @@
       </c>
       <c r="AL46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="AL47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -14326,7 +14326,7 @@
       </c>
       <c r="AL53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -15018,7 +15018,7 @@
       </c>
       <c r="AP3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -15936,9 +15936,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -15946,9 +15946,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
@@ -15956,9 +15956,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
@@ -16073,13 +16073,13 @@
       </c>
       <c r="AO8" s="7" t="inlineStr">
         <is>
-          <t>v058_tload_fp16_tile_state; v058_tload_tile_state; v058_tload_tstore_common_profiles
-Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_row1, s16_row0, s16_row1, s8_row0, s8_row1, u8_row0, u8_row1, u16_row0, u16_row1, s32_row0, s32_row1, u32_row0, u32_row1, zero_stride_rows.</t>
+          <t>v058_tload_fp16_tile_state; v058_tload_fp32_profiles; v058_tload_tile_state; v058_tload_tstore_common_profiles
+Automated current-ISA profile verification; evidence refs: fp32_8x32.</t>
         </is>
       </c>
       <c r="AP8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -16292,7 +16292,7 @@
       </c>
       <c r="AP9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -16579,19 +16579,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="P11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="Q11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -16604,9 +16604,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="U11" s="6" t="inlineStr">
@@ -16711,13 +16711,13 @@
       </c>
       <c r="AO11" s="7" t="inlineStr">
         <is>
-          <t>v058_shared_tlsu; v058_tload_tstore_common_profiles
-Automated current-ISA profile verification; evidence refs: shared_part_pe0, shared_part_pe1, shared_part_pe2, shared_part_pe3.</t>
+          <t>v058_shared_tlsu; v058_tload_tstore_common_profiles; v058_tstore_fp32_profiles; v058_tstore_s32_profile
+Automated current-ISA profile verification; evidence refs: store_s32_4x8.</t>
         </is>
       </c>
       <c r="AP11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -16987,7 +16987,7 @@
       </c>
       <c r="W2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17105,7 +17105,7 @@
       </c>
       <c r="W3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17223,7 +17223,7 @@
       </c>
       <c r="W4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17341,7 +17341,7 @@
       </c>
       <c r="W5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17459,7 +17459,7 @@
       </c>
       <c r="W6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17577,7 +17577,7 @@
       </c>
       <c r="W7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17690,12 +17690,12 @@
       <c r="V8" s="7" t="inlineStr">
         <is>
           <t>v058_cube_tmatmul_s32; v058_cube_tmatmul_shared_ab_fp32
-Automated current-ISA profile verification; evidence refs: shared_ab_tmatmul_fp32_m32_n32_k32.</t>
+Automated current-ISA profile verification; evidence refs: single_tmatmul_s32_m4_n8_k4_col8.</t>
         </is>
       </c>
       <c r="W8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17813,7 +17813,7 @@
       </c>
       <c r="W9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -17931,7 +17931,7 @@
       </c>
       <c r="W10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -18043,13 +18043,13 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>v058_cube_tmatmul_mx_e4m3
+          <t>v058_cube_tmatmul_mx_e2m1_hif4; v058_cube_tmatmul_mx_e4m3; v058_cube_tmatmul_mx_fp4_e2m1; v058_cube_tmatmul_mx_fp4_hif4; v058_cube_tmatmul_mx_hif4_e2m1
 Automated current-ISA profile verification; evidence refs: single_tmatmul_mx_e4m3_m4_n8_k4.</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -18167,7 +18167,7 @@
       </c>
       <c r="W12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -18285,7 +18285,7 @@
       </c>
       <c r="W13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qemu): refresh SFU profile matrix
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -241,17 +241,17 @@
         <v>222</v>
       </c>
       <c r="C8" s="3">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D8" s="4">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E8" s="5">
         <v>2</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>85.6%</t>
+          <t>86.5%</t>
         </is>
       </c>
     </row>
@@ -265,17 +265,17 @@
         <v>248</v>
       </c>
       <c r="C9" s="3">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D9" s="4">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E9" s="5">
         <v>21</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
@@ -337,17 +337,17 @@
         <v>546</v>
       </c>
       <c r="C12" s="3">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="D12" s="4">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="E12" s="5">
         <v>24</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>48.0%</t>
         </is>
       </c>
     </row>
@@ -1344,9 +1344,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1401,12 +1401,13 @@
       </c>
       <c r="S10" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_sfu_binary_unary_profiles
+Automated current-ISA profile verification; evidence refs: tdiv_s32.</t>
         </is>
       </c>
       <c r="T10" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2888,9 +2889,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -2945,12 +2946,13 @@
       </c>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>Zero divisors are data content, not an encoding/descriptor legality condition (TREM.md defines only element-wise remainder with divisor-signed remainder). QEMU no longer rejects divisor tiles containing 0; QEMU returns 0 for zero divisor while gfrun returns all-1s. ISA does not define the zero-divisor value, so the cell stays UNVERIFIED.</t>
+          <t>v058_tepl_sfu_binary_unary_profiles
+Automated current-ISA profile verification; evidence refs: trem_s32.</t>
         </is>
       </c>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -7654,9 +7656,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M19" s="6" t="inlineStr">
@@ -7781,12 +7783,13 @@
       </c>
       <c r="AK19" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_sfu_binary_unary_profiles
+Automated current-ISA profile verification; evidence refs: texp_f32.</t>
         </is>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -9002,9 +9005,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -9129,12 +9132,13 @@
       </c>
       <c r="AK26" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_sfu_binary_unary_profiles
+Automated current-ISA profile verification; evidence refs: tlog_f32.</t>
         </is>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -10348,9 +10352,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M33" s="6" t="inlineStr">
@@ -10475,12 +10479,13 @@
       </c>
       <c r="AK33" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_sfu_binary_unary_profiles
+Automated current-ISA profile verification; evidence refs: trecip_f32.</t>
         </is>
       </c>
       <c r="AL33" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -13233,9 +13238,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M48" s="6" t="inlineStr">
@@ -13360,12 +13365,13 @@
       </c>
       <c r="AK48" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_sfu_binary_unary_profiles
+Automated current-ISA profile verification; evidence refs: trsqr_f32.</t>
         </is>
       </c>
       <c r="AL48" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -13809,9 +13815,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L51" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M51" s="6" t="inlineStr">
@@ -13936,12 +13942,13 @@
       </c>
       <c r="AK51" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_sfu_binary_unary_profiles
+Automated current-ISA profile verification; evidence refs: tsqrt_f32.</t>
         </is>
       </c>
       <c r="AL51" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(qemu): align row arg-reduction with ASL
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -265,17 +265,17 @@
         <v>248</v>
       </c>
       <c r="C9" s="3">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D9" s="4">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E9" s="5">
         <v>21</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
@@ -337,17 +337,17 @@
         <v>546</v>
       </c>
       <c r="C12" s="3">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="D12" s="4">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="E12" s="5">
         <v>24</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>49.1%</t>
         </is>
       </c>
     </row>
@@ -7252,9 +7252,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -7399,12 +7399,13 @@
       </c>
       <c r="AK17" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_tconcat_s32
+Automated current-ISA profile verification; evidence refs: concat_s32.</t>
         </is>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -9371,9 +9372,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -9518,12 +9519,13 @@
       </c>
       <c r="AK28" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_tpart_s32
+Automated current-ISA profile verification; evidence refs: part_add_s32.</t>
         </is>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -9563,9 +9565,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -9710,12 +9712,13 @@
       </c>
       <c r="AK29" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_tpart_s32
+Automated current-ISA profile verification; evidence refs: part_max_s32.</t>
         </is>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -9755,9 +9758,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -9902,12 +9905,13 @@
       </c>
       <c r="AK30" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_tpart_s32
+Automated current-ISA profile verification; evidence refs: part_min_s32.</t>
         </is>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -9947,9 +9951,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -10094,12 +10098,13 @@
       </c>
       <c r="AK31" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_tpart_s32
+Automated current-ISA profile verification; evidence refs: part_mul_s32.</t>
         </is>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -10565,9 +10570,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P34" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
@@ -10672,12 +10677,13 @@
       </c>
       <c r="AK34" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_trowargmax_f32
+Automated current-ISA profile verification; evidence refs: trowargmax_f32.</t>
         </is>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qemu): refresh current profile matrix
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -262,10 +262,10 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C9" s="3">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D9" s="4">
         <v>186</v>
@@ -275,7 +275,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
@@ -334,10 +334,10 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C12" s="3">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D12" s="4">
         <v>254</v>
@@ -347,7 +347,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>49.1%</t>
+          <t>49.2%</t>
         </is>
       </c>
     </row>
@@ -8023,9 +8023,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -8170,12 +8170,13 @@
       </c>
       <c r="AK21" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tepl_tfillpad_s32
+Automated current-ISA profile verification; evidence refs: fillpad_s32.</t>
         </is>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qemu): refresh current tile profile matrix
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -241,17 +241,17 @@
         <v>223</v>
       </c>
       <c r="C8" s="3">
-        <v>194</v>
+        <v>223</v>
       </c>
       <c r="D8" s="4">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E8" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>87.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -262,20 +262,20 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C9" s="3">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D9" s="4">
         <v>169</v>
       </c>
       <c r="E9" s="5">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>26.1%</t>
+          <t>27.6%</t>
         </is>
       </c>
     </row>
@@ -286,20 +286,20 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C10" s="3">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="D10" s="4">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>39.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -334,20 +334,20 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="C12" s="3">
-        <v>297</v>
+        <v>362</v>
       </c>
       <c r="D12" s="4">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="E12" s="5">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>53.3%</t>
+          <t>64.3%</t>
         </is>
       </c>
     </row>
@@ -1267,19 +1267,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P9" s="6" t="inlineStr">
@@ -1299,12 +1299,13 @@
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>QEMU TCVT now accepts B.DATR PadValue (Zero/Max/Min/Null) per B.DATR.md PadValue table; the previous TEPL DATR gate rejected PadValue on TCVT. 91-case rerun: tmov/tcvt/cast_back*/expand_to_mhc_bwd/fused_weight/reduce_fused/swiglu PASS. Cell stays UNVERIFIED because bin ELFs are regression material, not independent numeric golden.</t>
+          <t>v058_tcvt_a5_profiles; v058_tcvt_fp8_probe; v058_tcvt_source_shape
+Automated current-ISA profile verification; evidence refs: f16_to_e4m3.</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1334,14 +1335,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1349,14 +1350,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1364,9 +1365,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
@@ -1401,8 +1402,8 @@
       </c>
       <c r="S10" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_sfu_binary_unary_profiles
-Automated current-ISA profile verification; evidence refs: tdiv_s32.</t>
+          <t>v058_tepl_sfu_binary_unary_profiles; v058_tepl_tdiv_trem_profiles
+Automated current-ISA profile verification; evidence refs: tdiv_f32.</t>
         </is>
       </c>
       <c r="T10" s="7" t="inlineStr">
@@ -1530,49 +1531,49 @@
           <t>tile-scalar-and-immediate-initialization</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M12" s="6" t="inlineStr">
@@ -1608,7 +1609,7 @@
       <c r="S12" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expands_profiles
-Automated current-ISA profile verification; evidence refs: texpands_u8, texpands_s8, texpands_u16, texpands_s16, texpands_u32, texpands_s32, texpands_f16, texpands_bf16, texpands_f32.</t>
+Automated current-ISA profile verification; evidence refs: texpands_f32.</t>
         </is>
       </c>
       <c r="T12" s="7" t="inlineStr">
@@ -1663,14 +1664,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>UNSUPPORTED</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>UNSUPPORTED</t>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1710,8 +1711,8 @@
       </c>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_tfma_f32
-Automated current-ISA profile verification; evidence refs: tfma_f32.</t>
+          <t>v058_tepl_tfma_bf16; v058_tepl_tfma_f16; v058_tepl_tfma_f32
+Automated current-ISA profile verification; evidence refs: tfma_bf16.</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
@@ -2879,14 +2880,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -2894,14 +2895,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
@@ -2909,9 +2910,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -2946,8 +2947,8 @@
       </c>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_sfu_binary_unary_profiles
-Automated current-ISA profile verification; evidence refs: trem_s32.</t>
+          <t>v058_tepl_sfu_binary_unary_profiles; v058_tepl_tdiv_trem_profiles
+Automated current-ISA profile verification; evidence refs: trem_f32.</t>
         </is>
       </c>
       <c r="T25" s="7" t="inlineStr">
@@ -2982,14 +2983,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -2997,14 +2998,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -3012,9 +3013,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -3049,8 +3050,8 @@
       </c>
       <c r="S26" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_trems_s32
-Automated current-ISA profile verification; evidence refs: trems_s32.</t>
+          <t>v058_tepl_trems_profiles; v058_tepl_trems_s32
+Automated current-ISA profile verification; evidence refs: trems_f32.</t>
         </is>
       </c>
       <c r="T26" s="7" t="inlineStr">
@@ -4142,8 +4143,11 @@
     <col min="41" max="41" width="14" customWidth="1"/>
     <col min="42" max="42" width="14" customWidth="1"/>
     <col min="43" max="43" width="14" customWidth="1"/>
-    <col min="44" max="44" width="58" customWidth="1"/>
+    <col min="44" max="44" width="14" customWidth="1"/>
     <col min="45" max="45" width="14" customWidth="1"/>
+    <col min="46" max="46" width="14" customWidth="1"/>
+    <col min="47" max="47" width="58" customWidth="1"/>
+    <col min="48" max="48" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4269,105 +4273,120 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>FP32 -&gt; S8; RNE; default multiplier 1.0 and zero point 0</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>FP4(e2m1x2/e1m2x2)</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FP8(e4m3/e5m2)</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FP8(e5m2/e4m3/e8m0)</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>HiF8</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>INT8: F32 -&gt; S8/U8; MXFP8: F32/BF16/F16 -&gt; FP8(e4m3); MXFP4: BF16/F16 -&gt; FP4(e2m1x2)</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>S/U16</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>S/U32/F32)</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>S32 value/index</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>S32/U32/S16/U16; ascending and descending; NORM row-major</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>S8 -&gt; FP32; RNE; default multiplier 1.0 and zero point 0</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>S8/U8/S16/U16/S32/U32/F16/BF16/F32; lower and upper; 4x4</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>U32; mask gather also S8</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>data: S32</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>index gather data: S16</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>indices: U32</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>source: U16</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>src/dst same dtype: S8</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>src: F16</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>src: S8</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>src: S8 or S16; dst/scale/offset: F32</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>values: source/destination dtype match</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Evidence / Notes</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -4529,9 +4548,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AF2" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AF2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AG2" s="6" t="inlineStr">
@@ -4539,9 +4558,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AH2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AI2" s="6" t="inlineStr">
@@ -4589,13 +4608,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR2" s="7" t="inlineStr">
+      <c r="AR2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU2" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tci_profiles
 Automated current-ISA profile verification; evidence refs: tci_s32_ascending, tci_u32_ascending, tci_s16_ascending, tci_u16_ascending, tci_s32_descending, tci_u32_descending, tci_s16_descending, tci_u16_descending.</t>
         </is>
       </c>
-      <c r="AS2" s="7" t="inlineStr">
+      <c r="AV2" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -4802,28 +4836,43 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AO3" s="4" t="inlineStr">
+      <c r="AO3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AP3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AQ3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AR3" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AP3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AR3" s="7" t="inlineStr">
+      <c r="AS3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU3" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tcolarg_f32
 Automated current-ISA profile verification; evidence refs: tcolargmax_f32.</t>
         </is>
       </c>
-      <c r="AS3" s="7" t="inlineStr">
+      <c r="AV3" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -5030,28 +5079,43 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AO4" s="4" t="inlineStr">
+      <c r="AO4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AP4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AQ4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AR4" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AP4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AR4" s="7" t="inlineStr">
+      <c r="AS4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU4" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tcolarg_f32
 Automated current-ISA profile verification; evidence refs: tcolargmin_f32.</t>
         </is>
       </c>
-      <c r="AS4" s="7" t="inlineStr">
+      <c r="AV4" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -5273,13 +5337,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR5" s="7" t="inlineStr">
+      <c r="AR5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU5" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_copy
 Automated current-ISA profile verification; evidence refs: tcolexpand_f32.</t>
         </is>
       </c>
-      <c r="AS5" s="7" t="inlineStr">
+      <c r="AV5" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -5501,13 +5580,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR6" s="7" t="inlineStr">
+      <c r="AR6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU6" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: col_add.</t>
         </is>
       </c>
-      <c r="AS6" s="7" t="inlineStr">
+      <c r="AV6" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -5729,13 +5823,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR7" s="7" t="inlineStr">
+      <c r="AR7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU7" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: col_div.</t>
         </is>
       </c>
-      <c r="AS7" s="7" t="inlineStr">
+      <c r="AV7" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -5957,13 +6066,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR8" s="7" t="inlineStr">
+      <c r="AR8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU8" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expandexpdif_f32
 Automated current-ISA profile verification; evidence refs: col_expdif.</t>
         </is>
       </c>
-      <c r="AS8" s="7" t="inlineStr">
+      <c r="AV8" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -6185,13 +6309,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR9" s="7" t="inlineStr">
+      <c r="AR9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU9" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: col_max.</t>
         </is>
       </c>
-      <c r="AS9" s="7" t="inlineStr">
+      <c r="AV9" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -6413,13 +6552,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR10" s="7" t="inlineStr">
+      <c r="AR10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU10" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: col_min.</t>
         </is>
       </c>
-      <c r="AS10" s="7" t="inlineStr">
+      <c r="AV10" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -6641,13 +6795,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR11" s="7" t="inlineStr">
+      <c r="AR11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU11" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: col_mul.</t>
         </is>
       </c>
-      <c r="AS11" s="7" t="inlineStr">
+      <c r="AV11" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -6869,13 +7038,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR12" s="7" t="inlineStr">
+      <c r="AR12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU12" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: col_sub.</t>
         </is>
       </c>
-      <c r="AS12" s="7" t="inlineStr">
+      <c r="AV12" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -7097,13 +7281,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR13" s="7" t="inlineStr">
+      <c r="AR13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU13" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_reduce_f32_profiles
 Automated current-ISA profile verification; evidence refs: tcolmax_f32.</t>
         </is>
       </c>
-      <c r="AS13" s="7" t="inlineStr">
+      <c r="AV13" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -7325,13 +7524,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR14" s="7" t="inlineStr">
+      <c r="AR14" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS14" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT14" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU14" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_reduce_f32_profiles
 Automated current-ISA profile verification; evidence refs: tcolmin_f32.</t>
         </is>
       </c>
-      <c r="AS14" s="7" t="inlineStr">
+      <c r="AV14" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -7553,13 +7767,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR15" s="7" t="inlineStr">
+      <c r="AR15" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS15" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT15" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU15" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_reduce_f32_profiles
 Automated current-ISA profile verification; evidence refs: tcolprod_f32.</t>
         </is>
       </c>
-      <c r="AS15" s="7" t="inlineStr">
+      <c r="AV15" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -7781,13 +8010,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR16" s="7" t="inlineStr">
+      <c r="AR16" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS16" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT16" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU16" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_reduce_f32_profiles
 Automated current-ISA profile verification; evidence refs: tcolsum_f32.</t>
         </is>
       </c>
-      <c r="AS16" s="7" t="inlineStr">
+      <c r="AV16" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -8009,13 +8253,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR17" s="7" t="inlineStr">
+      <c r="AR17" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS17" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT17" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU17" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tconcat_s32
 Automated current-ISA profile verification; evidence refs: concat_s32.</t>
         </is>
       </c>
-      <c r="AS17" s="7" t="inlineStr">
+      <c r="AV17" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -8192,9 +8451,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI18" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AI18" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AJ18" s="6" t="inlineStr">
@@ -8227,24 +8486,40 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AP18" s="4" t="inlineStr">
+      <c r="AP18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AQ18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AR18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS18" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AQ18" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AR18" s="7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AS18" s="7" t="inlineStr">
-        <is>
-          <t/>
+      <c r="AT18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU18" s="7" t="inlineStr">
+        <is>
+          <t>v058_tepl_tdequant_s8
+Automated current-ISA profile verification; evidence refs: dequant_fp32.</t>
+        </is>
+      </c>
+      <c r="AV18" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -8464,13 +8739,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR19" s="7" t="inlineStr">
+      <c r="AR19" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS19" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT19" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU19" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sfu_binary_unary_profiles
 Automated current-ISA profile verification; evidence refs: texp_f32.</t>
         </is>
       </c>
-      <c r="AS19" s="7" t="inlineStr">
+      <c r="AV19" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -8597,31 +8887,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Y20" s="4" t="inlineStr">
+      <c r="Y20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z20" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="Z20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA20" s="4" t="inlineStr">
+      <c r="AA20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AB20" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AB20" s="4" t="inlineStr">
+      <c r="AC20" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AC20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AD20" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -8667,38 +8957,53 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AM20" s="4" t="inlineStr">
+      <c r="AM20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AP20" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AN20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AP20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AQ20" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR20" s="7" t="inlineStr">
+      <c r="AR20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU20" s="7" t="inlineStr">
         <is>
           <t>v058_irregular_layout_profiles
 Automated current-ISA profile verification; evidence refs: textract_fp32.</t>
         </is>
       </c>
-      <c r="AS20" s="7" t="inlineStr">
+      <c r="AV20" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -8850,21 +9155,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AD21" s="4" t="inlineStr">
+      <c r="AD21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE21" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AE21" s="4" t="inlineStr">
+      <c r="AF21" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AF21" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AG21" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -8920,13 +9225,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR21" s="7" t="inlineStr">
+      <c r="AR21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU21" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tfillpad_s32
 Automated current-ISA profile verification; evidence refs: fillpad_s32.</t>
         </is>
       </c>
-      <c r="AS21" s="7" t="inlineStr">
+      <c r="AV21" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -9058,26 +9378,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z22" s="4" t="inlineStr">
+      <c r="Z22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA22" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AA22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AB22" s="4" t="inlineStr">
+      <c r="AB22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AC22" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AC22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AD22" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -9093,41 +9413,41 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AG22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH22" s="4" t="inlineStr">
+      <c r="AG22" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AH22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AI22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK22" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AI22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ22" s="4" t="inlineStr">
+      <c r="AL22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM22" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AK22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AN22" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -9148,14 +9468,30 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR22" s="7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AS22" s="7" t="inlineStr">
-        <is>
-          <t/>
+      <c r="AR22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU22" s="7" t="inlineStr">
+        <is>
+          <t>v058_tepl_tgather_s32
+Automated current-ISA profile verification; evidence refs: gather_s32.</t>
+        </is>
+      </c>
+      <c r="AV22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -9345,26 +9681,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AL23" s="5" t="inlineStr">
+      <c r="AL23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO23" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="AM23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AP23" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -9375,13 +9711,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR23" s="7" t="inlineStr">
+      <c r="AR23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU23" s="7" t="inlineStr">
         <is>
           <t>v058_irregular_layout_profiles
 Automated current-ISA profile verification; evidence refs: thistogram_u32_byte3.</t>
         </is>
       </c>
-      <c r="AS23" s="7" t="inlineStr">
+      <c r="AV23" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -9603,13 +9954,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR24" s="7" t="inlineStr">
+      <c r="AR24" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS24" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT24" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU24" s="7" t="inlineStr">
         <is>
           <t>QEMU fail-closed support audit
 The current QEMU head rejects this identity/profile before destination mutation.</t>
         </is>
       </c>
-      <c r="AS24" s="7" t="inlineStr">
+      <c r="AV24" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -9651,195 +10017,210 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr">
+      <c r="L25" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr">
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="X25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Y25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z25" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="M25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="P25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="V25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Y25" s="5" t="inlineStr">
+      <c r="AA25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AB25" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="Z25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA25" s="5" t="inlineStr">
+      <c r="AC25" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="AB25" s="5" t="inlineStr">
+      <c r="AD25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AF25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AG25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AH25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AI25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AP25" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="AC25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AD25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AE25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM25" s="5" t="inlineStr">
-        <is>
-          <t>UNSUPPORTED</t>
-        </is>
-      </c>
-      <c r="AN25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AP25" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AQ25" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR25" s="7" t="inlineStr">
-        <is>
-          <t>QEMU fail-closed support audit
-The current QEMU head rejects this identity/profile before destination mutation.</t>
-        </is>
-      </c>
-      <c r="AS25" s="7" t="inlineStr">
-        <is>
-          <t/>
+      <c r="AR25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU25" s="7" t="inlineStr">
+        <is>
+          <t>v058_tepl_tinsert_s32
+Automated current-ISA profile verification; evidence refs: insert_s32.</t>
+        </is>
+      </c>
+      <c r="AV25" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -10059,13 +10440,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR26" s="7" t="inlineStr">
+      <c r="AR26" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS26" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT26" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU26" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sfu_binary_unary_profiles
 Automated current-ISA profile verification; evidence refs: tlog_f32.</t>
         </is>
       </c>
-      <c r="AS26" s="7" t="inlineStr">
+      <c r="AV26" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -10287,13 +10683,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR27" s="7" t="inlineStr">
+      <c r="AR27" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS27" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT27" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU27" s="7" t="inlineStr">
         <is>
           <t>QEMU fail-closed support audit
 The current QEMU head rejects this identity/profile before destination mutation.</t>
         </is>
       </c>
-      <c r="AS27" s="7" t="inlineStr">
+      <c r="AV27" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -10515,13 +10926,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR28" s="7" t="inlineStr">
+      <c r="AR28" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS28" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT28" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU28" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tpart_s32
 Automated current-ISA profile verification; evidence refs: part_add_s32.</t>
         </is>
       </c>
-      <c r="AS28" s="7" t="inlineStr">
+      <c r="AV28" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -10743,13 +11169,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR29" s="7" t="inlineStr">
+      <c r="AR29" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS29" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT29" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU29" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tpart_s32
 Automated current-ISA profile verification; evidence refs: part_max_s32.</t>
         </is>
       </c>
-      <c r="AS29" s="7" t="inlineStr">
+      <c r="AV29" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -10971,13 +11412,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR30" s="7" t="inlineStr">
+      <c r="AR30" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS30" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT30" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU30" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tpart_s32
 Automated current-ISA profile verification; evidence refs: part_min_s32.</t>
         </is>
       </c>
-      <c r="AS30" s="7" t="inlineStr">
+      <c r="AV30" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -11199,13 +11655,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR31" s="7" t="inlineStr">
+      <c r="AR31" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS31" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT31" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU31" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tpart_s32
 Automated current-ISA profile verification; evidence refs: part_mul_s32.</t>
         </is>
       </c>
-      <c r="AS31" s="7" t="inlineStr">
+      <c r="AV31" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -11332,9 +11803,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Y32" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="Y32" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="Z32" s="6" t="inlineStr">
@@ -11352,16 +11823,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AC32" s="5" t="inlineStr">
+      <c r="AC32" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AD32" s="5" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
-      <c r="AD32" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AE32" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -11427,15 +11898,30 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR32" s="7" t="inlineStr">
-        <is>
-          <t>QEMU fail-closed support audit
-The current QEMU head rejects this identity/profile before destination mutation.</t>
-        </is>
-      </c>
-      <c r="AS32" s="7" t="inlineStr">
-        <is>
-          <t/>
+      <c r="AR32" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS32" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT32" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU32" s="7" t="inlineStr">
+        <is>
+          <t>v058_tepl_tquant_s8
+Automated current-ISA profile verification; evidence refs: quant_s8.</t>
+        </is>
+      </c>
+      <c r="AV32" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -11655,13 +12141,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR33" s="7" t="inlineStr">
+      <c r="AR33" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS33" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT33" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU33" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sfu_binary_unary_profiles
 Automated current-ISA profile verification; evidence refs: trecip_f32.</t>
         </is>
       </c>
-      <c r="AS33" s="7" t="inlineStr">
+      <c r="AV33" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -11863,33 +12364,48 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AN34" s="4" t="inlineStr">
+      <c r="AN34" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO34" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AP34" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AQ34" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AO34" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AP34" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ34" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AR34" s="7" t="inlineStr">
+      <c r="AR34" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS34" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT34" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU34" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_trowargmax_f32
 Automated current-ISA profile verification; evidence refs: trowargmax_f32.</t>
         </is>
       </c>
-      <c r="AS34" s="7" t="inlineStr">
+      <c r="AV34" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -12091,33 +12607,48 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AN35" s="4" t="inlineStr">
+      <c r="AN35" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO35" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AP35" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AQ35" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AO35" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AP35" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ35" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AR35" s="7" t="inlineStr">
+      <c r="AR35" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS35" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT35" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU35" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_trowargmin_f32
 Automated current-ISA profile verification; evidence refs: trowargmin_f32.</t>
         </is>
       </c>
-      <c r="AS35" s="7" t="inlineStr">
+      <c r="AV35" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -12339,13 +12870,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR36" s="7" t="inlineStr">
+      <c r="AR36" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS36" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT36" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU36" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_copy
 Automated current-ISA profile verification; evidence refs: trowexpand_f32.</t>
         </is>
       </c>
-      <c r="AS36" s="7" t="inlineStr">
+      <c r="AV36" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -12567,13 +13113,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR37" s="7" t="inlineStr">
+      <c r="AR37" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS37" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT37" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU37" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: row_add.</t>
         </is>
       </c>
-      <c r="AS37" s="7" t="inlineStr">
+      <c r="AV37" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -12795,13 +13356,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR38" s="7" t="inlineStr">
+      <c r="AR38" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS38" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT38" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU38" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: row_div.</t>
         </is>
       </c>
-      <c r="AS38" s="7" t="inlineStr">
+      <c r="AV38" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -13023,13 +13599,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR39" s="7" t="inlineStr">
+      <c r="AR39" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS39" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT39" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU39" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expandexpdif_f32
 Automated current-ISA profile verification; evidence refs: row_expdif.</t>
         </is>
       </c>
-      <c r="AS39" s="7" t="inlineStr">
+      <c r="AV39" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -13251,13 +13842,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR40" s="7" t="inlineStr">
+      <c r="AR40" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS40" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT40" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU40" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: row_max.</t>
         </is>
       </c>
-      <c r="AS40" s="7" t="inlineStr">
+      <c r="AV40" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -13479,13 +14085,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR41" s="7" t="inlineStr">
+      <c r="AR41" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS41" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT41" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU41" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: row_min.</t>
         </is>
       </c>
-      <c r="AS41" s="7" t="inlineStr">
+      <c r="AV41" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -13707,13 +14328,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR42" s="7" t="inlineStr">
+      <c r="AR42" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS42" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT42" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU42" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: row_mul.</t>
         </is>
       </c>
-      <c r="AS42" s="7" t="inlineStr">
+      <c r="AV42" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -13935,13 +14571,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR43" s="7" t="inlineStr">
+      <c r="AR43" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS43" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT43" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU43" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_expand_f32
 Automated current-ISA profile verification; evidence refs: row_sub.</t>
         </is>
       </c>
-      <c r="AS43" s="7" t="inlineStr">
+      <c r="AV43" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -14163,13 +14814,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR44" s="7" t="inlineStr">
+      <c r="AR44" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS44" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT44" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU44" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_trowmax_u16
 Automated current-ISA profile verification; evidence refs: trowmax_u16.</t>
         </is>
       </c>
-      <c r="AS44" s="7" t="inlineStr">
+      <c r="AV44" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -14391,13 +15057,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR45" s="7" t="inlineStr">
+      <c r="AR45" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS45" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT45" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU45" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_reduce_f32_profiles
 Automated current-ISA profile verification; evidence refs: trowmin_f32.</t>
         </is>
       </c>
-      <c r="AS45" s="7" t="inlineStr">
+      <c r="AV45" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -14619,13 +15300,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR46" s="7" t="inlineStr">
+      <c r="AR46" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS46" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT46" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU46" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_reduce_f32_profiles
 Automated current-ISA profile verification; evidence refs: trowprod_f32.</t>
         </is>
       </c>
-      <c r="AS46" s="7" t="inlineStr">
+      <c r="AV46" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -14847,13 +15543,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR47" s="7" t="inlineStr">
+      <c r="AR47" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS47" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT47" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU47" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_reduce_f32_profiles
 Automated current-ISA profile verification; evidence refs: trowsum_f32.</t>
         </is>
       </c>
-      <c r="AS47" s="7" t="inlineStr">
+      <c r="AV47" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -15075,13 +15786,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR48" s="7" t="inlineStr">
+      <c r="AR48" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS48" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT48" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU48" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sfu_binary_unary_profiles
 Automated current-ISA profile verification; evidence refs: trsqr_f32.</t>
         </is>
       </c>
-      <c r="AS48" s="7" t="inlineStr">
+      <c r="AV48" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -15248,9 +15974,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AG49" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AG49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AH49" s="6" t="inlineStr">
@@ -15258,26 +15984,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI49" s="4" t="inlineStr">
+      <c r="AI49" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AJ49" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK49" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL49" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AJ49" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK49" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL49" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AM49" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -15303,14 +16029,30 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR49" s="7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AS49" s="7" t="inlineStr">
-        <is>
-          <t/>
+      <c r="AR49" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS49" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT49" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU49" s="7" t="inlineStr">
+        <is>
+          <t>v058_tepl_tscatter_s32
+Automated current-ISA profile verification; evidence refs: scatter_s32.</t>
+        </is>
+      </c>
+      <c r="AV49" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -15495,26 +16237,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK50" s="4" t="inlineStr">
+      <c r="AK50" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AL50" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AM50" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AN50" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AL50" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM50" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN50" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="AO50" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -15525,18 +16267,33 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AQ50" s="4" t="inlineStr">
+      <c r="AQ50" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AR50" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS50" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT50" s="4" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="AR50" s="7" t="inlineStr">
+      <c r="AU50" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_tsort
 Automated current-ISA profile verification; evidence refs: bf16_desc_values, bf16_desc_indices.</t>
         </is>
       </c>
-      <c r="AS50" s="7" t="inlineStr">
+      <c r="AV50" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -15758,13 +16515,28 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR51" s="7" t="inlineStr">
+      <c r="AR51" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS51" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT51" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU51" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_sfu_binary_unary_profiles
 Automated current-ISA profile verification; evidence refs: tsqrt_f32.</t>
         </is>
       </c>
-      <c r="AS51" s="7" t="inlineStr">
+      <c r="AV51" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
@@ -15986,12 +16758,27 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR52" s="7" t="inlineStr">
+      <c r="AR52" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS52" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT52" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU52" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="AS52" s="7" t="inlineStr">
+      <c r="AV52" s="7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -16158,9 +16945,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AG53" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AG53" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AH53" s="6" t="inlineStr">
@@ -16173,9 +16960,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ53" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AJ53" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK53" s="6" t="inlineStr">
@@ -16213,20 +17000,35 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AR53" s="7" t="inlineStr">
+      <c r="AR53" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS53" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT53" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AU53" s="7" t="inlineStr">
         <is>
           <t>v058_tepl_ttri_profiles
 Automated current-ISA profile verification; evidence refs: ttri_s32_lower, ttri_u32_lower, ttri_s16_lower, ttri_u16_lower, ttri_s8_lower, ttri_u8_lower, ttri_f16_lower, ttri_bf16_lower, ttri_f32_lower, ttri_s32_upper, ttri_u32_upper, ttri_s16_upper, ttri_u16_upper, ttri_s8_upper, ttri_u8_upper, ttri_f16_upper, ttri_bf16_upper, ttri_f32_upper.</t>
         </is>
       </c>
-      <c r="AS53" s="7" t="inlineStr">
+      <c r="AV53" s="7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AS53"/>
+  <autoFilter ref="A1:AV53"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -16677,9 +17479,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AL2" s="5" t="inlineStr">
-        <is>
-          <t>UNSUPPORTED</t>
+      <c r="AL2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AM2" s="6" t="inlineStr">
@@ -16694,13 +17496,13 @@
       </c>
       <c r="AO2" s="7" t="inlineStr">
         <is>
-          <t>QEMU fail-closed support audit
-The current QEMU head rejects this identity/profile before destination mutation.</t>
+          <t>v058_tlsu_gmov_4pe
+Automated current-ISA profile verification; evidence refs: pe0, pe1, pe2, pe3.</t>
         </is>
       </c>
       <c r="AP2" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -16720,9 +17522,9 @@
           <t>memory-and-data-movement-irregular</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -16730,19 +17532,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -16750,19 +17552,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
@@ -16900,15 +17702,15 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AN3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AN3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AO3" s="7" t="inlineStr">
         <is>
-          <t>v058_irregular_layout_profiles
-Automated current-ISA profile verification; evidence refs: mgather_u32.</t>
+          <t>v058_tlsu_mgather_profiles
+Automated current-ISA profile verification; evidence refs: gather_f32.</t>
         </is>
       </c>
       <c r="AP3" s="7" t="inlineStr">
@@ -17083,9 +17885,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AH4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AI4" s="6" t="inlineStr">
@@ -17120,12 +17922,13 @@
       </c>
       <c r="AO4" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tlsu_mgather_cas_s32
+Automated current-ISA profile verification; evidence refs: mgather_cas_s32.</t>
         </is>
       </c>
       <c r="AP4" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -17165,9 +17968,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -17300,9 +18103,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AI5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AJ5" s="6" t="inlineStr">
@@ -17332,12 +18135,13 @@
       </c>
       <c r="AO5" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tlsu_mgather_mask_profiles; v058_tlsu_mgather_mask_s32
+Automated current-ISA profile verification; evidence refs: gather_u8, gather_s8, gather_u16, gather_s16, gather_u32, gather_s32, gather_f16, gather_bf16, gather_f32.</t>
         </is>
       </c>
       <c r="AP5" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -17362,44 +18166,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -17532,9 +18336,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AM6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AM6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AN6" s="6" t="inlineStr">
@@ -17544,12 +18348,13 @@
       </c>
       <c r="AO6" s="7" t="inlineStr">
         <is>
-          <t>Source-only stores accept TSize=000 and derive size from the source descriptor per B.IOT.md; index dtype gate enforces S32/U32 per MSCATTER.md and fails closed before memory side effects. 91-case rerun: mscatter_i32 PASS; mscatter_fp16/fp32 FAIL_ILLEGAL because their index tile dtype is FP16/FP32. Cell stays UNVERIFIED without an independent golden.</t>
+          <t>v058_tlsu_mscatter_profiles
+Automated current-ISA profile verification; evidence refs: scatter_f32.</t>
         </is>
       </c>
       <c r="AP6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -17589,9 +18394,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -17729,9 +18534,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ7" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AJ7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK7" s="6" t="inlineStr">
@@ -17756,12 +18561,13 @@
       </c>
       <c r="AO7" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>v058_tlsu_mscatter_mask_profiles; v058_tlsu_mscatter_mask_s32
+Automated current-ISA profile verification; evidence refs: scatter_u8, scatter_s8, scatter_u16, scatter_s16, scatter_u32, scatter_s32, scatter_f16, scatter_bf16, scatter_f32.</t>
         </is>
       </c>
       <c r="AP7" s="7" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -17866,9 +18672,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="V8" s="6" t="inlineStr">
@@ -17901,24 +18707,24 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AB8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AC8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AD8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="AE8" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AB8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AF8" s="6" t="inlineStr">
@@ -17968,8 +18774,8 @@
       </c>
       <c r="AO8" s="7" t="inlineStr">
         <is>
-          <t>v058_tload_fp16_tile_state; v058_tload_fp32_profiles; v058_tload_tile_state; v058_tload_tstore_common_profiles
-Automated current-ISA profile verification; evidence refs: fp32_8x32.</t>
+          <t>v058_tload_fp16_tile_state; v058_tload_fp32_profiles; v058_tload_shared_pe0_fp32_k16n32; v058_tload_shared_pe0_fp32_k32n16; v058_tload_shared_pe0_fp32_k32n32; v058_tload_shared_pe0_s8; v058_tload_tile_state; v058_tload_tstore_common_profiles
+Automated current-ISA profile verification; evidence refs: valid, pad.</t>
         </is>
       </c>
       <c r="AP8" s="7" t="inlineStr">
@@ -18159,9 +18965,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK9" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AK9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL9" s="6" t="inlineStr">
@@ -18181,8 +18987,8 @@
       </c>
       <c r="AO9" s="7" t="inlineStr">
         <is>
-          <t>v058_tmov_shared_fp32
-Automated current-ISA profile verification; evidence refs: publish_extract_pe0, publish_extract_pe1, publish_extract_pe2, publish_extract_pe3.</t>
+          <t>v058_tmov; v058_tmov_shared_fp32
+Automated current-ISA profile verification; evidence refs: tmov_s32.</t>
         </is>
       </c>
       <c r="AP9" s="7" t="inlineStr">
@@ -18302,9 +19108,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="W10" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="W10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="X10" s="6" t="inlineStr">
@@ -18510,9 +19316,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="V11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="V11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="W11" s="6" t="inlineStr">
@@ -18608,7 +19414,7 @@
       <c r="AO11" s="7" t="inlineStr">
         <is>
           <t>v058_shared_tlsu; v058_tload_tstore_common_profiles; v058_tstore_fp32_profiles; v058_tstore_s32_profile
-Automated current-ISA profile verification; evidence refs: store_s32_4x8.</t>
+Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_gap0, fp32_row1, fp32_tail, s16_row0, s16_gap, s16_row1, s16_tail, s8_row0, s8_gap, s8_row1, s8_tail, u8_row0, u8_gap, u8_row1, u8_tail, u16_row0, u16_gap, u16_row1, u16_tail, s32_row0, s32_gap, s32_row1, s32_tail, u32_row0, u32_gap, u32_row1, u32_tail, zero_stride_rows, zero_stride_tail.</t>
         </is>
       </c>
       <c r="AP11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs(status): refresh QEMU CUBE profile matrix after ASL repartition
Regenerate the QEMU tile profile workbook from the SuperScalarModel status
whose CUBE profiles are partitioned by ASL numeric class (Float->F32,
Signed->S32, Unsigned->U32, plus MX no-scale/with-scale).
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -310,20 +310,20 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C11" s="3">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D11" s="4">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="E11" s="5">
         <v>0</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>58.6%</t>
+          <t>24.1%</t>
         </is>
       </c>
     </row>
@@ -334,20 +334,20 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>563</v>
+        <v>588</v>
       </c>
       <c r="C12" s="3">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="D12" s="4">
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="E12" s="5">
         <v>20</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>64.3%</t>
+          <t>60.9%</t>
         </is>
       </c>
     </row>
@@ -19476,92 +19476,92 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</t>
+          <t>Local Float matrix pair -&gt; F32</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Local E2M1X2xE2M1X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+          <t>Local Float matrix/vector -&gt; F32</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Local E2M1X2xHiF4X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+          <t>Local MX E4M3/E5M2/E2M1X2/E1M2X2 matrix/vector (E8M0 scale) -&gt; F32</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Local E4M3 matrix/vector with E8M0 scales + scalar FP32 bias -&gt; F32; M4N1K4</t>
+          <t>Local MX E4M3/E5M2/E2M1X2/E1M2X2 pair (E8M0 scale) -&gt; F32</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Local E4M3 matrix/vector with E8M0 scales -&gt; F32; M4N1K4; Col8</t>
+          <t>Local MX FP16/BF16 matrix/vector (no scale) -&gt; F32</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Local E4M3xE4M3 with E8M0 scales + FP32 row bias -&gt; F32; M4N8K4</t>
+          <t>Local MX FP16/BF16 pair (no scale) -&gt; F32</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Local E4M3xE4M3 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+          <t>Local Signed matrix pair -&gt; S32</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Local HiF4X2xE2M1X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+          <t>Local Signed matrix/vector -&gt; S32</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Local HiF4X2xHiF4X2 with E8M0 scales -&gt; F32; NORM; M4N8K4; Col8</t>
+          <t>Local Unsigned matrix pair -&gt; U32</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Local S32 matrix x S32 vector + scalar S32 bias -&gt; S32; M4N1K4</t>
+          <t>Local Unsigned matrix/vector -&gt; U32</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Local S32 matrix x S32 vector -&gt; S32; NORM; M4N1K4; Col8</t>
+          <t>Shared Both Float matrix pair -&gt; F32</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Local S32xS32 + row-bias S32 -&gt; S32; NORM; M4N8K4; Col8</t>
+          <t>Shared Both MX pair -&gt; F32</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Local S32xS32 -&gt; S32; NORM row-major; M4N8K4; Col8; 256B D</t>
+          <t>Shared Both Signed matrix pair -&gt; S32</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Local explicit C S32 + S32xS32 -&gt; S32 D; NORM; M4N8K4; Col8</t>
+          <t>Shared Both Unsigned matrix pair -&gt; U32</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Local explicit FP32 C + E4M3 matrix/vector with E8M0 scales -&gt; F32 D; M4N1K4</t>
+          <t>Shared Right Float matrix pair -&gt; F32</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Local explicit FP32 C + E4M3xE4M3 with E8M0 scales -&gt; F32 D; M4N8K4</t>
+          <t>Shared Right MX pair -&gt; F32</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Local explicit S32 C + S32 matrix x vector -&gt; S32 D; M4N1K4; Col8</t>
+          <t>Shared Right Signed matrix pair -&gt; S32</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Shared Left F32xF32 + Shared Right F32xF32 -&gt; Local F32 D; NORM; Core4; M=N=K=32; 4KB per PE</t>
+          <t>Shared Right Unsigned matrix pair -&gt; U32</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -19591,14 +19591,14 @@
           <t>matrix-and-matrix-vector-matrix-vector</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -19626,9 +19626,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -19636,14 +19636,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O2" s="6" t="inlineStr">
@@ -19709,14 +19709,14 @@
           <t>matrix-and-matrix-vector-matrix-vector</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -19744,9 +19744,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -19754,9 +19754,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="N3" s="6" t="inlineStr">
@@ -19789,9 +19789,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="T3" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U3" s="6" t="inlineStr">
@@ -19827,14 +19827,14 @@
           <t>matrix-and-matrix-vector-matrix-vector</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -19862,9 +19862,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -19872,9 +19872,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -19945,9 +19945,9 @@
           <t>matrix-and-matrix-vector-matrix-vector</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -19955,9 +19955,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -19965,9 +19965,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -20063,9 +20063,9 @@
           <t>matrix-and-matrix-vector-matrix-vector</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -20073,9 +20073,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -20083,9 +20083,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -20133,9 +20133,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
@@ -20181,9 +20181,9 @@
           <t>matrix-and-matrix-vector-matrix-vector</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -20191,19 +20191,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -20329,9 +20329,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -20339,9 +20339,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -20349,9 +20349,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -20359,19 +20359,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="Q8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="S8" s="6" t="inlineStr">
@@ -20379,14 +20379,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="T8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="V8" s="7" t="inlineStr">
@@ -20447,9 +20447,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -20457,9 +20457,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
@@ -20467,9 +20467,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -20477,19 +20477,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="R9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="S9" s="6" t="inlineStr">
@@ -20497,14 +20497,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="T9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
@@ -20565,9 +20565,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -20575,9 +20575,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
@@ -20585,29 +20585,29 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O10" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="S10" s="6" t="inlineStr">
@@ -20615,14 +20615,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="V10" s="7" t="inlineStr">
@@ -20653,24 +20653,24 @@
           <t>matrix-and-matrix-vector-matrix-matrix</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -20678,24 +20678,24 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
@@ -20708,9 +20708,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="P11" s="6" t="inlineStr">
@@ -20728,9 +20728,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="T11" s="6" t="inlineStr">
@@ -20771,9 +20771,9 @@
           <t>matrix-and-matrix-vector-matrix-matrix</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -20786,9 +20786,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -20796,9 +20796,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -20826,9 +20826,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="P12" s="6" t="inlineStr">
@@ -20846,9 +20846,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S12" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="T12" s="6" t="inlineStr">
@@ -20889,9 +20889,9 @@
           <t>matrix-and-matrix-vector-matrix-matrix</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -20904,9 +20904,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -20914,9 +20914,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -20944,9 +20944,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="P13" s="6" t="inlineStr">
@@ -20964,9 +20964,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="S13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="T13" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(status): refresh QEMU CUBE matrix after gfrun dtype promotion
Regenerate the QEMU CUBE profile matrix after the SuperScalarModel
cross-model status promoted the ordinary TMATMUL Local Float/Unsigned
class profiles on gfrun.  QEMU stays UNVERIFIED for those two classes
because the current QEMU CUBE path cannot execute any v058 CUBE block.
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -170,7 +170,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="T2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="T3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="T4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="T10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="T20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="T22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2747,7 +2747,7 @@
       </c>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="T24" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="T26" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="T30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="T32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="T34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4086,7 +4086,7 @@
       </c>
       <c r="T36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="AV2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AV3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="AV4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="AV5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="AV6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -5846,7 +5846,7 @@
       </c>
       <c r="AV7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="AV8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6332,7 @@
       </c>
       <c r="AV9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="AV10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AV11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7061,7 +7061,7 @@
       </c>
       <c r="AV12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="AV13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7547,7 @@
       </c>
       <c r="AV14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7790,7 +7790,7 @@
       </c>
       <c r="AV15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="AV16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -8276,7 +8276,7 @@
       </c>
       <c r="AV17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -8519,7 +8519,7 @@
       </c>
       <c r="AV18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -8762,7 +8762,7 @@
       </c>
       <c r="AV19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -9005,7 +9005,7 @@
       </c>
       <c r="AV20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AV21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -9491,7 +9491,7 @@
       </c>
       <c r="AV22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -9734,7 +9734,7 @@
       </c>
       <c r="AV23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="AV25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -10463,7 +10463,7 @@
       </c>
       <c r="AV26" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -10949,7 +10949,7 @@
       </c>
       <c r="AV28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -11192,7 +11192,7 @@
       </c>
       <c r="AV29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -11435,7 +11435,7 @@
       </c>
       <c r="AV30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -11678,7 +11678,7 @@
       </c>
       <c r="AV31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -11921,7 +11921,7 @@
       </c>
       <c r="AV32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -12164,7 +12164,7 @@
       </c>
       <c r="AV33" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -12407,7 +12407,7 @@
       </c>
       <c r="AV34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -12650,7 +12650,7 @@
       </c>
       <c r="AV35" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -12893,7 +12893,7 @@
       </c>
       <c r="AV36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -13136,7 +13136,7 @@
       </c>
       <c r="AV37" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -13379,7 +13379,7 @@
       </c>
       <c r="AV38" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -13622,7 +13622,7 @@
       </c>
       <c r="AV39" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -13865,7 +13865,7 @@
       </c>
       <c r="AV40" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -14108,7 +14108,7 @@
       </c>
       <c r="AV41" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -14351,7 +14351,7 @@
       </c>
       <c r="AV42" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -14594,7 +14594,7 @@
       </c>
       <c r="AV43" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -14837,7 +14837,7 @@
       </c>
       <c r="AV44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -15080,7 +15080,7 @@
       </c>
       <c r="AV45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -15323,7 +15323,7 @@
       </c>
       <c r="AV46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -15566,7 +15566,7 @@
       </c>
       <c r="AV47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -15809,7 +15809,7 @@
       </c>
       <c r="AV48" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -16052,7 +16052,7 @@
       </c>
       <c r="AV49" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -16295,7 +16295,7 @@
       </c>
       <c r="AV50" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -16538,7 +16538,7 @@
       </c>
       <c r="AV51" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -17023,7 +17023,7 @@
       </c>
       <c r="AV53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -17502,7 +17502,7 @@
       </c>
       <c r="AP2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -17715,7 +17715,7 @@
       </c>
       <c r="AP3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -17928,7 +17928,7 @@
       </c>
       <c r="AP4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -18141,7 +18141,7 @@
       </c>
       <c r="AP5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -18354,7 +18354,7 @@
       </c>
       <c r="AP6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -18567,7 +18567,7 @@
       </c>
       <c r="AP7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -18780,7 +18780,7 @@
       </c>
       <c r="AP8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -18993,7 +18993,7 @@
       </c>
       <c r="AP9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -19206,7 +19206,7 @@
       </c>
       <c r="AP10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -19419,7 +19419,7 @@
       </c>
       <c r="AP11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -19689,7 +19689,7 @@
       </c>
       <c r="W2" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -19807,7 +19807,7 @@
       </c>
       <c r="W3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -19925,7 +19925,7 @@
       </c>
       <c r="W4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20043,7 +20043,7 @@
       </c>
       <c r="W5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20161,7 +20161,7 @@
       </c>
       <c r="W6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20279,7 +20279,7 @@
       </c>
       <c r="W7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20391,13 +20391,13 @@
       </c>
       <c r="V8" s="7" t="inlineStr">
         <is>
-          <t>v058_cube_tmatmul_s32; v058_cube_tmatmul_shared_ab_fp32
+          <t>v058_cube_tmatmul_bf16; v058_cube_tmatmul_s32; v058_cube_tmatmul_shared_ab_fp32; v058_cube_tmatmul_u16
 Automated current-ISA profile verification; evidence refs: single_tmatmul_s32_m4_n8_k4_col8.</t>
         </is>
       </c>
       <c r="W8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20515,7 +20515,7 @@
       </c>
       <c r="W9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20633,7 +20633,7 @@
       </c>
       <c r="W10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20751,7 +20751,7 @@
       </c>
       <c r="W11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20869,7 +20869,7 @@
       </c>
       <c r="W12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -20987,7 +20987,7 @@
       </c>
       <c r="W13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(qemu): align v058 cross-model contracts
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support.xlsx
@@ -241,17 +241,17 @@
         <v>223</v>
       </c>
       <c r="C8" s="3">
-        <v>223</v>
+        <v>209</v>
       </c>
       <c r="D8" s="4">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E8" s="5">
         <v>0</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>93.7%</t>
         </is>
       </c>
     </row>
@@ -265,17 +265,17 @@
         <v>261</v>
       </c>
       <c r="C9" s="3">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D9" s="4">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E9" s="5">
         <v>20</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>26.8%</t>
         </is>
       </c>
     </row>
@@ -286,10 +286,10 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C10" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D10" s="4">
         <v>0</v>
@@ -334,20 +334,20 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C12" s="3">
-        <v>358</v>
+        <v>338</v>
       </c>
       <c r="D12" s="4">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="E12" s="5">
         <v>20</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>60.9%</t>
+          <t>57.9%</t>
         </is>
       </c>
     </row>
@@ -1016,29 +1016,29 @@
           <t>elementwise-tile-tile-logical</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -1046,9 +1046,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -1056,9 +1056,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
@@ -1081,9 +1081,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -1093,13 +1093,12 @@
       </c>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_compare_byte_float_profiles; v058_tepl_compare_integer_profiles
-Automated current-ISA profile verification; evidence refs: tcmp_u16_gt.</t>
+          <t>Automated current-ISA profile verification; evidence refs: tcmp_u16_gt.</t>
         </is>
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
@@ -1129,14 +1128,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1149,9 +1148,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -1159,9 +1158,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -1179,9 +1178,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="P8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
@@ -1196,13 +1195,12 @@
       </c>
       <c r="S8" s="7" t="inlineStr">
         <is>
-          <t>v058_tepl_compare_scalar_modes; v058_tepl_compare_scalar_profiles
-Automated current-ISA profile verification; evidence refs: tcmps_u16_gt.</t>
+          <t>Automated current-ISA profile verification; evidence refs: tcmps_u16_gt.</t>
         </is>
       </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
@@ -1272,9 +1270,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1299,13 +1297,13 @@
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>v058_tcvt_a5_profiles; v058_tcvt_fp8_probe; v058_tcvt_source_shape
+          <t>v058_tcvt_a5_profiles; v058_tcvt_fp8_probe
 Automated current-ISA profile verification; evidence refs: f16_to_e4m3.</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
@@ -8822,9 +8820,9 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
@@ -8999,13 +8997,12 @@
       </c>
       <c r="AU20" s="7" t="inlineStr">
         <is>
-          <t>v058_irregular_layout_profiles
-Automated current-ISA profile verification; evidence refs: textract_fp32.</t>
+          <t>Automated current-ISA profile verification; evidence refs: textract_fp32.</t>
         </is>
       </c>
       <c r="AV20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
@@ -9536,9 +9533,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -9728,13 +9725,12 @@
       </c>
       <c r="AU23" s="7" t="inlineStr">
         <is>
-          <t>v058_irregular_layout_profiles
-Automated current-ISA profile verification; evidence refs: thistogram_u32_byte3.</t>
+          <t>Automated current-ISA profile verification; evidence refs: thistogram_u32_byte3.</t>
         </is>
       </c>
       <c r="AV23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
@@ -17073,12 +17069,8 @@
     <col min="34" max="34" width="14" customWidth="1"/>
     <col min="35" max="35" width="14" customWidth="1"/>
     <col min="36" max="36" width="14" customWidth="1"/>
-    <col min="37" max="37" width="14" customWidth="1"/>
+    <col min="37" max="37" width="58" customWidth="1"/>
     <col min="38" max="38" width="14" customWidth="1"/>
-    <col min="39" max="39" width="14" customWidth="1"/>
-    <col min="40" max="40" width="14" customWidth="1"/>
-    <col min="41" max="41" width="58" customWidth="1"/>
-    <col min="42" max="42" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17199,95 +17191,75 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Shared FP32; Function 10 L2S PUBLISH; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+          <t>Shared full FP32; PE0 issuer; K16xN32 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Shared FP32; Function 11 S2L BROADCAST; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+          <t>Shared full FP32; PE0 issuer; K32xN16 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Shared FP32; Function 12 S2L EXTRACT; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+          <t>Shared full FP32; PE0 issuer; K32xN32 NORM; PE-local 4KiB class 6; Core4 aggregate 16KiB</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Shared FP32; Function 9 L2S INSERT; PE_MASK 1111; PE-local 128B; NORM 4x8</t>
+          <t>Shared full S8; PE0 issuer; K16xN32 NORM; PE-local 512B class 3; Core4 aggregate 2KiB</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Shared full FP32; PE0 issuer; K16xN32 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
+          <t>Shared full/core FP32; B.IOS source; Function 1; NORM</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Shared full FP32; PE0 issuer; K32xN16 NORM; PE-local 2KiB class 5; Core4 aggregate 8KiB</t>
+          <t>Shared pe_scope FP32; B.IOS source; Function 14; NORM</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Shared full FP32; PE0 issuer; K32xN32 NORM; PE-local 4KiB class 6; Core4 aggregate 16KiB</t>
+          <t>TLSU atomic data types accepted by BSTART.MGATHER.CAS</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Shared full S8; PE0 issuer; K16xN32 NORM; PE-local 512B class 3; Core4 aggregate 2KiB</t>
+          <t>TLSU data types accepted by BSTART.MGATHER.MASK</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Shared full/core FP32; B.IOS source; Function 1; NORM</t>
+          <t>TLSU data types accepted by BSTART.MSCATTER.MASK</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Shared pe_scope FP32; B.IOS source; Function 14; NORM</t>
+          <t>byte-preserving; descriptors must be compatible</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>TLSU atomic data types accepted by BSTART.MGATHER.CAS</t>
+          <t>byte-preserving; source and destination descriptors must match</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>TLSU data types accepted by BSTART.MGATHER.MASK</t>
+          <t>data: S8</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>TLSU data types accepted by BSTART.MSCATTER.MASK</t>
+          <t>data: U8</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>byte-preserving; descriptors must be compatible</t>
+          <t>Evidence / Notes</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>byte-preserving; source and destination descriptors must match</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>data: S8</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>data: U8</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence / Notes</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
@@ -17459,9 +17431,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AH2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AI2" s="6" t="inlineStr">
@@ -17474,33 +17446,13 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL2" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AM2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN2" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO2" s="7" t="inlineStr">
+      <c r="AK2" s="7" t="inlineStr">
         <is>
           <t>v058_tlsu_gmov_4pe
 Automated current-ISA profile verification; evidence refs: pe0, pe1, pe2, pe3.</t>
         </is>
       </c>
-      <c r="AP2" s="7" t="inlineStr">
+      <c r="AL2" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -17682,38 +17634,18 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM3" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN3" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AO3" s="7" t="inlineStr">
+      <c r="AJ3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AK3" s="7" t="inlineStr">
         <is>
           <t>v058_tlsu_mgather_profiles
 Automated current-ISA profile verification; evidence refs: gather_f32.</t>
         </is>
       </c>
-      <c r="AP3" s="7" t="inlineStr">
+      <c r="AL3" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -17865,9 +17797,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AD4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AE4" s="6" t="inlineStr">
@@ -17885,9 +17817,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH4" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AH4" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AI4" s="6" t="inlineStr">
@@ -17900,33 +17832,13 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN4" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO4" s="7" t="inlineStr">
+      <c r="AK4" s="7" t="inlineStr">
         <is>
           <t>v058_tlsu_mgather_cas_s32
 Automated current-ISA profile verification; evidence refs: mgather_cas_s32.</t>
         </is>
       </c>
-      <c r="AP4" s="7" t="inlineStr">
+      <c r="AL4" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -18083,9 +17995,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AE5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AE5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AF5" s="6" t="inlineStr">
@@ -18103,9 +18015,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI5" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AI5" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AJ5" s="6" t="inlineStr">
@@ -18113,33 +18025,13 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN5" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO5" s="7" t="inlineStr">
+      <c r="AK5" s="7" t="inlineStr">
         <is>
           <t>v058_tlsu_mgather_mask_profiles; v058_tlsu_mgather_mask_s32
 Automated current-ISA profile verification; evidence refs: gather_u8, gather_s8, gather_u16, gather_s16, gather_u32, gather_s32, gather_f16, gather_bf16, gather_f32.</t>
         </is>
       </c>
-      <c r="AP5" s="7" t="inlineStr">
+      <c r="AL5" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -18316,9 +18208,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AI6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AI6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AJ6" s="6" t="inlineStr">
@@ -18326,33 +18218,13 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM6" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AN6" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO6" s="7" t="inlineStr">
+      <c r="AK6" s="7" t="inlineStr">
         <is>
           <t>v058_tlsu_mscatter_profiles
 Automated current-ISA profile verification; evidence refs: scatter_f32.</t>
         </is>
       </c>
-      <c r="AP6" s="7" t="inlineStr">
+      <c r="AL6" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -18514,9 +18386,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AF7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AF7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AG7" s="6" t="inlineStr">
@@ -18534,38 +18406,18 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AJ7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AK7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN7" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO7" s="7" t="inlineStr">
+      <c r="AJ7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AK7" s="7" t="inlineStr">
         <is>
           <t>v058_tlsu_mscatter_mask_profiles; v058_tlsu_mscatter_mask_s32
 Automated current-ISA profile verification; evidence refs: scatter_u8, scatter_s8, scatter_u16, scatter_s16, scatter_u32, scatter_s32, scatter_f16, scatter_bf16, scatter_f32.</t>
         </is>
       </c>
-      <c r="AP7" s="7" t="inlineStr">
+      <c r="AL7" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -18687,44 +18539,44 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="X8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Y8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Z8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AB8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AC8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AD8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AE8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="X8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AC8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AD8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AF8" s="6" t="inlineStr">
@@ -18752,33 +18604,13 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN8" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO8" s="7" t="inlineStr">
+      <c r="AK8" s="7" t="inlineStr">
         <is>
           <t>v058_tload_fp16_tile_state; v058_tload_fp32_profiles; v058_tload_shared_pe0_fp32_k16n32; v058_tload_shared_pe0_fp32_k32n16; v058_tload_shared_pe0_fp32_k32n32; v058_tload_shared_pe0_s8; v058_tload_tile_state; v058_tload_tstore_common_profiles
 Automated current-ISA profile verification; evidence refs: valid, pad.</t>
         </is>
       </c>
-      <c r="AP8" s="7" t="inlineStr">
+      <c r="AL8" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -18900,24 +18732,24 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="X9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="Y9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="Z9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AA9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Y9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AB9" s="6" t="inlineStr">
@@ -18945,9 +18777,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AG9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AG9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AH9" s="6" t="inlineStr">
@@ -18965,33 +18797,13 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AL9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO9" s="7" t="inlineStr">
-        <is>
-          <t>v058_tmov; v058_tmov_shared_fp32
+      <c r="AK9" s="7" t="inlineStr">
+        <is>
+          <t>v058_tmov
 Automated current-ISA profile verification; evidence refs: tmov_s32.</t>
         </is>
       </c>
-      <c r="AP9" s="7" t="inlineStr">
+      <c r="AL9" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -19178,33 +18990,13 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO10" s="7" t="inlineStr">
+      <c r="AK10" s="7" t="inlineStr">
         <is>
           <t>v058_tlsu_tprefetch_s32
 Automated current-ISA profile verification; evidence refs: prefetch_s32.</t>
         </is>
       </c>
-      <c r="AP10" s="7" t="inlineStr">
+      <c r="AL10" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -19346,14 +19138,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AB11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AC11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="AB11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AD11" s="6" t="inlineStr">
@@ -19366,14 +19158,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AF11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AG11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="AF11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AG11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AH11" s="6" t="inlineStr">
@@ -19391,40 +19183,20 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AK11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AL11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AM11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AN11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AO11" s="7" t="inlineStr">
+      <c r="AK11" s="7" t="inlineStr">
         <is>
           <t>v058_shared_tlsu; v058_tload_tstore_common_profiles; v058_tstore_fp32_profiles; v058_tstore_s32_profile
 Automated current-ISA profile verification; evidence refs: fp32_row0, fp32_gap0, fp32_row1, fp32_tail, s16_row0, s16_gap, s16_row1, s16_tail, s8_row0, s8_gap, s8_row1, s8_tail, u8_row0, u8_gap, u8_row1, u8_tail, u16_row0, u16_gap, u16_row1, u16_tail, s32_row0, s32_gap, s32_row1, s32_tail, u32_row0, u32_gap, u32_row1, u32_tail, zero_stride_rows, zero_stride_tail.</t>
         </is>
       </c>
-      <c r="AP11" s="7" t="inlineStr">
+      <c r="AL11" s="7" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP11"/>
+  <autoFilter ref="A1:AL11"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>